<commit_message>
seo: internal links to alphabet guide, GSC evidence in core
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8056" uniqueCount="922">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8075" uniqueCount="927">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
@@ -2326,6 +2326,15 @@
     <t>priority_score confidence: low | needs volume — editorial seed keyword, zero provider or GSC evidence yet; Volume queried 2026-10-14 (DataForSEO Google Ads Search Volume): no data available (&lt;10/mo or unrated); SERP validated 2026-10-14 (US/en, mobile Android, top 10 organic): 7 organic results; no HebrewEdu URL in top 10</t>
   </si>
   <si>
+    <t>hebrew alphabet</t>
+  </si>
+  <si>
+    <t>GSC (owner-reported, 2026-10-14)</t>
+  </si>
+  <si>
+    <t>GSC evidence, 28-day window pulled 2026-10-14 (impressions began 2026-10-10): 213 impressions, avg position ~11, 0 clicks, for https://hebrewedu.com/blog/hebrew-alphabet-complete-guide/. Not the same window as this file's gsc_impr_3m/gsc_pos_3m (3-month) columns, left blank here rather than merged. No paid SERP call made for this exact keyword; gap analysis instead uses the 2026-10-14 DataForSEO batch's top-10 organic for the same cluster's SERP-validated proxies (hebrew alphabet chart, hebrew alphabet course, hebrew alphabet pronunciation) — see docs/seo/alphabet-guide-gap-2026-10-14.md.</t>
+  </si>
+  <si>
     <t>url</t>
   </si>
   <si>
@@ -2428,7 +2437,13 @@
     <t>Everything you need to know about the Hebrew alphabet — letter shapes, names, sounds, and practical tips for learning Aleph Bet from scratch.</t>
   </si>
   <si>
-    <t>how many letters are in the hebrew alphabet; hebrew alphabet pronunciation; how to read hebrew; learn hebrew alphabet; learning the hebrew alphabet; learn aleph bet; alephbet; hebrew alphabet letter names; hebrew final letters; hebrew reading direction; learn hebrew alphabet online; how to pronounce chet in hebrew; how to pronounce resh in hebrew; hebrew capital and lowercase letters; bet vs vet pronunciation; shin vs sin pronunciation; kaf vs chaf pronunciation; vav vowel and consonant sounds; yod vowel and consonant sounds; learn hebrew aleph bet; learning hebrew alphabet; learn hebrew letters; learn hebrew alef bet; how to learn hebrew alphabet; hebrew aleph bet; learn hebrew script; learning hebrew letters; aleph bet; hebrew alef bet; how to learn hebrew letters; aleph bet hebrew; easy way to learn hebrew alphabet; hebrew alphabet learn</t>
+    <t>hebrew alphabet; how many letters are in the hebrew alphabet; hebrew alphabet pronunciation; how to read hebrew; learn hebrew alphabet; learning the hebrew alphabet; learn aleph bet; alephbet; hebrew alphabet letter names; hebrew final letters; hebrew reading direction; learn hebrew alphabet online; how to pronounce chet in hebrew; how to pronounce resh in hebrew; hebrew capital and lowercase letters; bet vs vet pronunciation; shin vs sin pronunciation; kaf vs chaf pronunciation; vav vowel and consonant sounds; yod vowel and consonant sounds; learn hebrew aleph bet; learning hebrew alphabet; learn hebrew letters; learn hebrew alef bet; how to learn hebrew alphabet; hebrew aleph bet; learn hebrew script; learning hebrew letters; aleph bet; hebrew alef bet; how to learn hebrew letters; aleph bet hebrew; easy way to learn hebrew alphabet; hebrew alphabet learn</t>
+  </si>
+  <si>
+    <t>213</t>
+  </si>
+  <si>
+    <t>2026-10-10 export (page-baseline.csv); hebrew alphabet query, GSC last 28 days pulled 2026-10-14 (impressions began 2026-10-10)</t>
   </si>
   <si>
     <t>What Are Hebrew Binyanim? A Practical Beginner's Guide | HebrewEdu Blog</t>
@@ -2770,19 +2785,19 @@
     <t>max_priority_score</t>
   </si>
   <si>
-    <t>224/352 keywords have no recorded search volume.</t>
-  </si>
-  <si>
-    <t>253/352 keywords have no recorded keyword difficulty.</t>
-  </si>
-  <si>
-    <t>264/352 keywords are not yet SERP-validated (serp_validated != yes).</t>
-  </si>
-  <si>
-    <t>43/352 keywords are still status=candidate (not promoted).</t>
-  </si>
-  <si>
-    <t>349/352 keywords have no rank_baseline_pos on record.</t>
+    <t>225/353 keywords have no recorded search volume.</t>
+  </si>
+  <si>
+    <t>254/353 keywords have no recorded keyword difficulty.</t>
+  </si>
+  <si>
+    <t>265/353 keywords are not yet SERP-validated (serp_validated != yes).</t>
+  </si>
+  <si>
+    <t>43/353 keywords are still status=candidate (not promoted).</t>
+  </si>
+  <si>
+    <t>350/353 keywords have no rank_baseline_pos on record.</t>
   </si>
 </sst>
 </file>
@@ -5481,7 +5496,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S353"/>
+  <dimension ref="A1:S354"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -26323,6 +26338,65 @@
       </c>
       <c r="S353" t="s">
         <v>768</v>
+      </c>
+    </row>
+    <row r="354" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A354" t="s">
+        <v>769</v>
+      </c>
+      <c r="B354" t="s">
+        <v>302</v>
+      </c>
+      <c r="C354" t="s">
+        <v>2</v>
+      </c>
+      <c r="D354" t="s">
+        <v>2</v>
+      </c>
+      <c r="E354" t="s">
+        <v>2</v>
+      </c>
+      <c r="F354" t="s">
+        <v>2</v>
+      </c>
+      <c r="G354" t="s">
+        <v>343</v>
+      </c>
+      <c r="H354" t="s">
+        <v>23</v>
+      </c>
+      <c r="I354" t="s">
+        <v>312</v>
+      </c>
+      <c r="J354" t="s">
+        <v>28</v>
+      </c>
+      <c r="K354" t="s">
+        <v>306</v>
+      </c>
+      <c r="L354" t="s">
+        <v>29</v>
+      </c>
+      <c r="M354" t="s">
+        <v>312</v>
+      </c>
+      <c r="N354" t="s">
+        <v>2</v>
+      </c>
+      <c r="O354" t="s">
+        <v>2</v>
+      </c>
+      <c r="P354" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q354" t="s">
+        <v>353</v>
+      </c>
+      <c r="R354" t="s">
+        <v>770</v>
+      </c>
+      <c r="S354" t="s">
+        <v>771</v>
       </c>
     </row>
   </sheetData>
@@ -26352,28 +26426,28 @@
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>773</v>
+        <v>776</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>775</v>
+        <v>778</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>296</v>
@@ -26382,16 +26456,16 @@
         <v>297</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>777</v>
+        <v>780</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>778</v>
+        <v>781</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>20</v>
@@ -26402,13 +26476,13 @@
         <v>87</v>
       </c>
       <c r="B2" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="C2" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="D2" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="E2" t="s">
         <v>83</v>
@@ -26417,28 +26491,28 @@
         <v>317</v>
       </c>
       <c r="G2" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
       <c r="H2" t="s">
         <v>386</v>
       </c>
       <c r="I2" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="J2" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
       <c r="K2" t="s">
         <v>107</v>
       </c>
       <c r="L2" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="M2" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="N2" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O2" t="s">
         <v>29</v>
@@ -26446,16 +26520,16 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="B3" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="C3" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
       <c r="D3" t="s">
-        <v>792</v>
+        <v>795</v>
       </c>
       <c r="E3" t="s">
         <v>2</v>
@@ -26470,10 +26544,10 @@
         <v>80</v>
       </c>
       <c r="I3" t="s">
-        <v>793</v>
+        <v>796</v>
       </c>
       <c r="J3" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="K3" t="s">
         <v>80</v>
@@ -26482,10 +26556,10 @@
         <v>715</v>
       </c>
       <c r="M3" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="N3" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O3" t="s">
         <v>29</v>
@@ -26496,13 +26570,13 @@
         <v>183</v>
       </c>
       <c r="B4" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="C4" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="D4" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="E4" t="s">
         <v>180</v>
@@ -26511,7 +26585,7 @@
         <v>663</v>
       </c>
       <c r="G4" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
       <c r="H4" t="s">
         <v>2</v>
@@ -26532,7 +26606,7 @@
         <v>2</v>
       </c>
       <c r="N4" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O4" t="s">
         <v>29</v>
@@ -26543,13 +26617,13 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="C5" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="D5" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
       <c r="E5" t="s">
         <v>23</v>
@@ -26558,7 +26632,7 @@
         <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="H5" t="s">
         <v>2</v>
@@ -26570,16 +26644,16 @@
         <v>2</v>
       </c>
       <c r="K5" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="L5" t="s">
-        <v>2</v>
+        <v>807</v>
       </c>
       <c r="M5" t="s">
-        <v>2</v>
+        <v>492</v>
       </c>
       <c r="N5" t="s">
-        <v>788</v>
+        <v>808</v>
       </c>
       <c r="O5" t="s">
         <v>29</v>
@@ -26590,13 +26664,13 @@
         <v>194</v>
       </c>
       <c r="B6" t="s">
-        <v>804</v>
+        <v>809</v>
       </c>
       <c r="C6" t="s">
-        <v>805</v>
+        <v>810</v>
       </c>
       <c r="D6" t="s">
-        <v>806</v>
+        <v>811</v>
       </c>
       <c r="E6" t="s">
         <v>191</v>
@@ -26605,7 +26679,7 @@
         <v>193</v>
       </c>
       <c r="G6" t="s">
-        <v>807</v>
+        <v>812</v>
       </c>
       <c r="H6" t="s">
         <v>2</v>
@@ -26626,7 +26700,7 @@
         <v>2</v>
       </c>
       <c r="N6" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O6" t="s">
         <v>29</v>
@@ -26637,13 +26711,13 @@
         <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>808</v>
+        <v>813</v>
       </c>
       <c r="C7" t="s">
-        <v>809</v>
+        <v>814</v>
       </c>
       <c r="D7" t="s">
-        <v>810</v>
+        <v>815</v>
       </c>
       <c r="E7" t="s">
         <v>56</v>
@@ -26652,7 +26726,7 @@
         <v>58</v>
       </c>
       <c r="G7" t="s">
-        <v>811</v>
+        <v>816</v>
       </c>
       <c r="H7" t="s">
         <v>80</v>
@@ -26661,19 +26735,19 @@
         <v>491</v>
       </c>
       <c r="J7" t="s">
-        <v>812</v>
+        <v>817</v>
       </c>
       <c r="K7" t="s">
         <v>80</v>
       </c>
       <c r="L7" t="s">
-        <v>813</v>
+        <v>818</v>
       </c>
       <c r="M7" t="s">
-        <v>814</v>
+        <v>819</v>
       </c>
       <c r="N7" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O7" t="s">
         <v>29</v>
@@ -26684,13 +26758,13 @@
         <v>247</v>
       </c>
       <c r="B8" t="s">
-        <v>815</v>
+        <v>820</v>
       </c>
       <c r="C8" t="s">
-        <v>816</v>
+        <v>821</v>
       </c>
       <c r="D8" t="s">
-        <v>817</v>
+        <v>822</v>
       </c>
       <c r="E8" t="s">
         <v>245</v>
@@ -26699,7 +26773,7 @@
         <v>440</v>
       </c>
       <c r="G8" t="s">
-        <v>818</v>
+        <v>823</v>
       </c>
       <c r="H8" t="s">
         <v>2</v>
@@ -26720,7 +26794,7 @@
         <v>2</v>
       </c>
       <c r="N8" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O8" t="s">
         <v>29</v>
@@ -26731,13 +26805,13 @@
         <v>188</v>
       </c>
       <c r="B9" t="s">
-        <v>819</v>
+        <v>824</v>
       </c>
       <c r="C9" t="s">
-        <v>820</v>
+        <v>825</v>
       </c>
       <c r="D9" t="s">
-        <v>821</v>
+        <v>826</v>
       </c>
       <c r="E9" t="s">
         <v>185</v>
@@ -26746,7 +26820,7 @@
         <v>186</v>
       </c>
       <c r="G9" t="s">
-        <v>822</v>
+        <v>827</v>
       </c>
       <c r="H9" t="s">
         <v>2</v>
@@ -26767,7 +26841,7 @@
         <v>2</v>
       </c>
       <c r="N9" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O9" t="s">
         <v>29</v>
@@ -26778,13 +26852,13 @@
         <v>197</v>
       </c>
       <c r="B10" t="s">
-        <v>823</v>
+        <v>828</v>
       </c>
       <c r="C10" t="s">
-        <v>824</v>
+        <v>829</v>
       </c>
       <c r="D10" t="s">
-        <v>825</v>
+        <v>830</v>
       </c>
       <c r="E10" t="s">
         <v>195</v>
@@ -26793,7 +26867,7 @@
         <v>196</v>
       </c>
       <c r="G10" t="s">
-        <v>826</v>
+        <v>831</v>
       </c>
       <c r="H10" t="s">
         <v>2</v>
@@ -26814,7 +26888,7 @@
         <v>2</v>
       </c>
       <c r="N10" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O10" t="s">
         <v>29</v>
@@ -26825,13 +26899,13 @@
         <v>166</v>
       </c>
       <c r="B11" t="s">
-        <v>827</v>
+        <v>832</v>
       </c>
       <c r="C11" t="s">
-        <v>828</v>
+        <v>833</v>
       </c>
       <c r="D11" t="s">
-        <v>829</v>
+        <v>834</v>
       </c>
       <c r="E11" t="s">
         <v>162</v>
@@ -26840,7 +26914,7 @@
         <v>164</v>
       </c>
       <c r="G11" t="s">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="H11" t="s">
         <v>80</v>
@@ -26849,7 +26923,7 @@
         <v>318</v>
       </c>
       <c r="J11" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="K11" t="s">
         <v>80</v>
@@ -26861,7 +26935,7 @@
         <v>466</v>
       </c>
       <c r="N11" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O11" t="s">
         <v>29</v>
@@ -26872,13 +26946,13 @@
         <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>832</v>
+        <v>837</v>
       </c>
       <c r="C12" t="s">
-        <v>833</v>
+        <v>838</v>
       </c>
       <c r="D12" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="E12" t="s">
         <v>71</v>
@@ -26887,7 +26961,7 @@
         <v>73</v>
       </c>
       <c r="G12" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="H12" t="s">
         <v>2</v>
@@ -26908,7 +26982,7 @@
         <v>2</v>
       </c>
       <c r="N12" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O12" t="s">
         <v>29</v>
@@ -26919,13 +26993,13 @@
         <v>216</v>
       </c>
       <c r="B13" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="C13" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
       <c r="D13" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
       <c r="E13" t="s">
         <v>214</v>
@@ -26934,7 +27008,7 @@
         <v>352</v>
       </c>
       <c r="G13" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
       <c r="H13" t="s">
         <v>2</v>
@@ -26955,7 +27029,7 @@
         <v>2</v>
       </c>
       <c r="N13" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O13" t="s">
         <v>29</v>
@@ -26966,13 +27040,13 @@
         <v>143</v>
       </c>
       <c r="B14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="C14" t="s">
-        <v>841</v>
+        <v>846</v>
       </c>
       <c r="D14" t="s">
-        <v>842</v>
+        <v>847</v>
       </c>
       <c r="E14" t="s">
         <v>204</v>
@@ -26981,7 +27055,7 @@
         <v>205</v>
       </c>
       <c r="G14" t="s">
-        <v>843</v>
+        <v>848</v>
       </c>
       <c r="H14" t="s">
         <v>2</v>
@@ -27002,7 +27076,7 @@
         <v>2</v>
       </c>
       <c r="N14" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O14" t="s">
         <v>29</v>
@@ -27010,16 +27084,16 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B15" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="C15" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="D15" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
       <c r="E15" t="s">
         <v>2</v>
@@ -27049,7 +27123,7 @@
         <v>2</v>
       </c>
       <c r="N15" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O15" t="s">
         <v>29</v>
@@ -27060,13 +27134,13 @@
         <v>208</v>
       </c>
       <c r="B16" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
       <c r="C16" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="D16" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
       <c r="E16" t="s">
         <v>206</v>
@@ -27075,7 +27149,7 @@
         <v>207</v>
       </c>
       <c r="G16" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="H16" t="s">
         <v>2</v>
@@ -27096,7 +27170,7 @@
         <v>2</v>
       </c>
       <c r="N16" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O16" t="s">
         <v>29</v>
@@ -27107,13 +27181,13 @@
         <v>266</v>
       </c>
       <c r="B17" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
       <c r="C17" t="s">
-        <v>853</v>
+        <v>858</v>
       </c>
       <c r="D17" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
       <c r="E17" t="s">
         <v>263</v>
@@ -27143,7 +27217,7 @@
         <v>2</v>
       </c>
       <c r="N17" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O17" t="s">
         <v>29</v>
@@ -27154,13 +27228,13 @@
         <v>231</v>
       </c>
       <c r="B18" t="s">
-        <v>855</v>
+        <v>860</v>
       </c>
       <c r="C18" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="D18" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="E18" t="s">
         <v>229</v>
@@ -27190,7 +27264,7 @@
         <v>2</v>
       </c>
       <c r="N18" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O18" t="s">
         <v>29</v>
@@ -27201,13 +27275,13 @@
         <v>223</v>
       </c>
       <c r="B19" t="s">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="C19" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="D19" t="s">
-        <v>860</v>
+        <v>865</v>
       </c>
       <c r="E19" t="s">
         <v>221</v>
@@ -27237,7 +27311,7 @@
         <v>2</v>
       </c>
       <c r="N19" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O19" t="s">
         <v>29</v>
@@ -27248,13 +27322,13 @@
         <v>127</v>
       </c>
       <c r="B20" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="C20" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
       <c r="D20" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="E20" t="s">
         <v>124</v>
@@ -27263,28 +27337,28 @@
         <v>125</v>
       </c>
       <c r="G20" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
       <c r="H20" t="s">
         <v>80</v>
       </c>
       <c r="I20" t="s">
-        <v>865</v>
+        <v>870</v>
       </c>
       <c r="J20" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="K20" t="s">
         <v>80</v>
       </c>
       <c r="L20" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="M20" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="N20" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O20" t="s">
         <v>29</v>
@@ -27295,13 +27369,13 @@
         <v>242</v>
       </c>
       <c r="B21" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="C21" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="D21" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
       <c r="E21" t="s">
         <v>240</v>
@@ -27310,7 +27384,7 @@
         <v>241</v>
       </c>
       <c r="G21" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="H21" t="s">
         <v>80</v>
@@ -27331,7 +27405,7 @@
         <v>529</v>
       </c>
       <c r="N21" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O21" t="s">
         <v>29</v>
@@ -27342,13 +27416,13 @@
         <v>179</v>
       </c>
       <c r="B22" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
       <c r="C22" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
       <c r="D22" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="E22" t="s">
         <v>175</v>
@@ -27357,7 +27431,7 @@
         <v>177</v>
       </c>
       <c r="G22" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="H22" t="s">
         <v>2</v>
@@ -27378,7 +27452,7 @@
         <v>2</v>
       </c>
       <c r="N22" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="O22" t="s">
         <v>29</v>
@@ -27389,13 +27463,13 @@
         <v>108</v>
       </c>
       <c r="B23" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="C23" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="D23" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="E23" t="s">
         <v>104</v>
@@ -27404,7 +27478,7 @@
         <v>105</v>
       </c>
       <c r="G23" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
       <c r="H23" t="s">
         <v>2</v>
@@ -27425,7 +27499,7 @@
         <v>2</v>
       </c>
       <c r="N23" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="O23" t="s">
         <v>29</v>
@@ -27436,13 +27510,13 @@
         <v>282</v>
       </c>
       <c r="B24" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
       <c r="C24" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
       <c r="D24" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="E24" t="s">
         <v>279</v>
@@ -27451,7 +27525,7 @@
         <v>755</v>
       </c>
       <c r="G24" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="H24" t="s">
         <v>2</v>
@@ -27472,7 +27546,7 @@
         <v>2</v>
       </c>
       <c r="N24" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="O24" t="s">
         <v>29</v>
@@ -27483,13 +27557,13 @@
         <v>203</v>
       </c>
       <c r="B25" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="C25" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="D25" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="E25" t="s">
         <v>201</v>
@@ -27498,7 +27572,7 @@
         <v>202</v>
       </c>
       <c r="G25" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="H25" t="s">
         <v>2</v>
@@ -27519,7 +27593,7 @@
         <v>2</v>
       </c>
       <c r="N25" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O25" t="s">
         <v>29</v>
@@ -27530,13 +27604,13 @@
         <v>171</v>
       </c>
       <c r="B26" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="C26" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="D26" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="E26" t="s">
         <v>167</v>
@@ -27545,7 +27619,7 @@
         <v>169</v>
       </c>
       <c r="G26" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="H26" t="s">
         <v>2</v>
@@ -27566,7 +27640,7 @@
         <v>2</v>
       </c>
       <c r="N26" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O26" t="s">
         <v>29</v>
@@ -27577,13 +27651,13 @@
         <v>228</v>
       </c>
       <c r="B27" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="C27" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="D27" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="E27" t="s">
         <v>256</v>
@@ -27592,7 +27666,7 @@
         <v>257</v>
       </c>
       <c r="G27" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="H27" t="s">
         <v>2</v>
@@ -27613,7 +27687,7 @@
         <v>2</v>
       </c>
       <c r="N27" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O27" t="s">
         <v>29</v>
@@ -27624,13 +27698,13 @@
         <v>286</v>
       </c>
       <c r="B28" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="C28" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="D28" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="E28" t="s">
         <v>283</v>
@@ -27639,7 +27713,7 @@
         <v>763</v>
       </c>
       <c r="G28" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
       <c r="H28" t="s">
         <v>2</v>
@@ -27660,7 +27734,7 @@
         <v>2</v>
       </c>
       <c r="N28" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="O28" t="s">
         <v>29</v>
@@ -27668,16 +27742,16 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="B29" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="C29" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="D29" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="E29" t="s">
         <v>2</v>
@@ -27695,7 +27769,7 @@
         <v>492</v>
       </c>
       <c r="J29" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="K29" t="s">
         <v>80</v>
@@ -27707,7 +27781,7 @@
         <v>64</v>
       </c>
       <c r="N29" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O29" t="s">
         <v>29</v>
@@ -27715,16 +27789,16 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="B30" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
       <c r="C30" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="D30" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="E30" t="s">
         <v>2</v>
@@ -27751,10 +27825,10 @@
         <v>95</v>
       </c>
       <c r="M30" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
       <c r="N30" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O30" t="s">
         <v>29</v>
@@ -27762,16 +27836,16 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="B31" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="C31" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
       <c r="D31" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="E31" t="s">
         <v>2</v>
@@ -27801,7 +27875,7 @@
         <v>2</v>
       </c>
       <c r="N31" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="O31" t="s">
         <v>29</v>
@@ -27843,7 +27917,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -28540,27 +28614,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
seo: alphabet guide FAQ from real PAA, faq field for blog posts
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -2329,10 +2329,10 @@
     <t>hebrew alphabet</t>
   </si>
   <si>
-    <t>GSC (owner-reported, 2026-10-14)</t>
-  </si>
-  <si>
-    <t>GSC evidence, 28-day window pulled 2026-10-14 (impressions began 2026-10-10): 213 impressions, avg position ~11, 0 clicks, for https://hebrewedu.com/blog/hebrew-alphabet-complete-guide/. Not the same window as this file's gsc_impr_3m/gsc_pos_3m (3-month) columns, left blank here rather than merged. No paid SERP call made for this exact keyword; gap analysis instead uses the 2026-10-14 DataForSEO batch's top-10 organic for the same cluster's SERP-validated proxies (hebrew alphabet chart, hebrew alphabet course, hebrew alphabet pronunciation) — see docs/seo/alphabet-guide-gap-2026-10-14.md.</t>
+    <t>DataForSEO SERP, research/semantic-core-v5-alphabet-faq/2026-10-14/serp_raw/00-hebrew-alphabet.json</t>
+  </si>
+  <si>
+    <t>GSC evidence, 28-day window pulled 2026-10-14 (impressions began 2026-10-10): 213 impressions, avg position ~11, 0 clicks, for https://hebrewedu.com/blog/hebrew-alphabet-complete-guide/. Not the same window as this file's gsc_impr_3m/gsc_pos_3m (3-month) columns, left blank here rather than merged. Direct SERP pull for this exact keyword done 2026-10-14 (US/en, mobile Android, depth 10, $0.002): organic is thin (6/10 slots; AI Overview, Images, Knowledge Graph and PAA outrank organic), no HebrewEdu URL present, no guide-style competitor in the top 6. PAA + Knowledge Graph panel questions from this pull were used to add an FAQ section to the guide — see docs/seo/alphabet-guide-gap-2026-10-14.md and research/semantic-core-v5-alphabet-faq/2026-10-14/serp_parsed.md.</t>
   </si>
   <si>
     <t>url</t>
@@ -2791,7 +2791,7 @@
     <t>254/353 keywords have no recorded keyword difficulty.</t>
   </si>
   <si>
-    <t>265/353 keywords are not yet SERP-validated (serp_validated != yes).</t>
+    <t>264/353 keywords are not yet SERP-validated (serp_validated != yes).</t>
   </si>
   <si>
     <t>43/353 keywords are still status=candidate (not promoted).</t>
@@ -26378,7 +26378,7 @@
         <v>29</v>
       </c>
       <c r="M354" t="s">
-        <v>312</v>
+        <v>30</v>
       </c>
       <c r="N354" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
lessons: publish Bet, editorial rules, keyword titles; csv eol=lf
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8075" uniqueCount="927">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8084" uniqueCount="931">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
@@ -2668,16 +2668,28 @@
     <t>no export covers this page yet</t>
   </si>
   <si>
-    <t>Aleph: three vowel marks | HebrewEdu</t>
-  </si>
-  <si>
-    <t>Exploring Aleph (א) and Hebrew Diacritical Marks</t>
-  </si>
-  <si>
-    <t>Exploring Aleph: The Foundation of the Hebrew Alphabet</t>
+    <t>Aleph Hebrew Letter (א): Vowel Marks</t>
+  </si>
+  <si>
+    <t>Aleph Hebrew Letter (א): Vowel Marks &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Aleph (א) and its three vowel marks — Patah, Kamatz Gadol and Hataf Patah — with beginner explanations and interactive practice.</t>
   </si>
   <si>
     <t>alef hebrew letter; hebrew aleph pronunciation; hebrew letter aleph sound; learn hebrew letter aleph; aleph hebrew letter exercises; aleph with patah; aleph with kamatz; aleph with hataf patah; is aleph silent</t>
+  </si>
+  <si>
+    <t>Bet Hebrew Letter (ב): Sound &amp; Dagesh</t>
+  </si>
+  <si>
+    <t>Bet Hebrew Letter (ב): Dagesh, Sound &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Bet (ב): how the dagesh dot changes its sound between [b] and [v], with beginner explanations, example words and interactive practice.</t>
+  </si>
+  <si>
+    <t>vet hebrew letter; hebrew bet pronunciation; hebrew letter bet sound; learn hebrew letter bet; bet hebrew letter exercises; bet with dagesh</t>
   </si>
   <si>
     <t>Hebrew Phrases for Beginners: 30 Useful Phrases | HebrewEdu</t>
@@ -3564,7 +3576,7 @@
         <v>70</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H10" t="s">
         <v>30</v>
@@ -14221,7 +14233,7 @@
         <v>306</v>
       </c>
       <c r="L148" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M148" t="s">
         <v>30</v>
@@ -14280,7 +14292,7 @@
         <v>306</v>
       </c>
       <c r="L149" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M149" t="s">
         <v>312</v>
@@ -14339,7 +14351,7 @@
         <v>306</v>
       </c>
       <c r="L150" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M150" t="s">
         <v>312</v>
@@ -14398,7 +14410,7 @@
         <v>306</v>
       </c>
       <c r="L151" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M151" t="s">
         <v>312</v>
@@ -14457,7 +14469,7 @@
         <v>306</v>
       </c>
       <c r="L152" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M152" t="s">
         <v>312</v>
@@ -14516,7 +14528,7 @@
         <v>306</v>
       </c>
       <c r="L153" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M153" t="s">
         <v>312</v>
@@ -14575,7 +14587,7 @@
         <v>306</v>
       </c>
       <c r="L154" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M154" t="s">
         <v>312</v>
@@ -26408,7 +26420,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -27507,7 +27519,7 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>282</v>
+        <v>70</v>
       </c>
       <c r="B24" t="s">
         <v>887</v>
@@ -27519,10 +27531,10 @@
         <v>889</v>
       </c>
       <c r="E24" t="s">
-        <v>279</v>
+        <v>66</v>
       </c>
       <c r="F24" t="s">
-        <v>755</v>
+        <v>67</v>
       </c>
       <c r="G24" t="s">
         <v>890</v>
@@ -27554,7 +27566,7 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>203</v>
+        <v>282</v>
       </c>
       <c r="B25" t="s">
         <v>891</v>
@@ -27566,10 +27578,10 @@
         <v>893</v>
       </c>
       <c r="E25" t="s">
-        <v>201</v>
+        <v>279</v>
       </c>
       <c r="F25" t="s">
-        <v>202</v>
+        <v>755</v>
       </c>
       <c r="G25" t="s">
         <v>894</v>
@@ -27593,7 +27605,7 @@
         <v>2</v>
       </c>
       <c r="N25" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O25" t="s">
         <v>29</v>
@@ -27601,7 +27613,7 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>171</v>
+        <v>203</v>
       </c>
       <c r="B26" t="s">
         <v>895</v>
@@ -27613,10 +27625,10 @@
         <v>897</v>
       </c>
       <c r="E26" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="F26" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="G26" t="s">
         <v>898</v>
@@ -27648,7 +27660,7 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>228</v>
+        <v>171</v>
       </c>
       <c r="B27" t="s">
         <v>899</v>
@@ -27660,10 +27672,10 @@
         <v>901</v>
       </c>
       <c r="E27" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="F27" t="s">
-        <v>257</v>
+        <v>169</v>
       </c>
       <c r="G27" t="s">
         <v>902</v>
@@ -27695,7 +27707,7 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>286</v>
+        <v>228</v>
       </c>
       <c r="B28" t="s">
         <v>903</v>
@@ -27707,10 +27719,10 @@
         <v>905</v>
       </c>
       <c r="E28" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F28" t="s">
-        <v>763</v>
+        <v>257</v>
       </c>
       <c r="G28" t="s">
         <v>906</v>
@@ -27734,7 +27746,7 @@
         <v>2</v>
       </c>
       <c r="N28" t="s">
-        <v>882</v>
+        <v>791</v>
       </c>
       <c r="O28" t="s">
         <v>29</v>
@@ -27742,46 +27754,46 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>286</v>
+      </c>
+      <c r="B29" t="s">
         <v>907</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>908</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>909</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
+        <v>283</v>
+      </c>
+      <c r="F29" t="s">
+        <v>763</v>
+      </c>
+      <c r="G29" t="s">
         <v>910</v>
       </c>
-      <c r="E29" t="s">
-        <v>2</v>
-      </c>
-      <c r="F29" t="s">
-        <v>2</v>
-      </c>
-      <c r="G29" t="s">
-        <v>2</v>
-      </c>
       <c r="H29" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I29" t="s">
-        <v>492</v>
+        <v>2</v>
       </c>
       <c r="J29" t="s">
-        <v>911</v>
+        <v>2</v>
       </c>
       <c r="K29" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="L29" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="M29" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N29" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O29" t="s">
         <v>29</v>
@@ -27789,16 +27801,16 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>911</v>
+      </c>
+      <c r="B30" t="s">
         <v>912</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>913</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>914</v>
-      </c>
-      <c r="D30" t="s">
-        <v>915</v>
       </c>
       <c r="E30" t="s">
         <v>2</v>
@@ -27813,19 +27825,19 @@
         <v>80</v>
       </c>
       <c r="I30" t="s">
-        <v>415</v>
+        <v>492</v>
       </c>
       <c r="J30" t="s">
-        <v>353</v>
+        <v>915</v>
       </c>
       <c r="K30" t="s">
         <v>80</v>
       </c>
       <c r="L30" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M30" t="s">
-        <v>916</v>
+        <v>64</v>
       </c>
       <c r="N30" t="s">
         <v>791</v>
@@ -27836,48 +27848,95 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>916</v>
+      </c>
+      <c r="B31" t="s">
         <v>917</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>918</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>919</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
+        <v>2</v>
+      </c>
+      <c r="F31" t="s">
+        <v>2</v>
+      </c>
+      <c r="G31" t="s">
+        <v>2</v>
+      </c>
+      <c r="H31" t="s">
+        <v>80</v>
+      </c>
+      <c r="I31" t="s">
+        <v>415</v>
+      </c>
+      <c r="J31" t="s">
+        <v>353</v>
+      </c>
+      <c r="K31" t="s">
+        <v>80</v>
+      </c>
+      <c r="L31" t="s">
+        <v>95</v>
+      </c>
+      <c r="M31" t="s">
         <v>920</v>
-      </c>
-      <c r="E31" t="s">
-        <v>2</v>
-      </c>
-      <c r="F31" t="s">
-        <v>2</v>
-      </c>
-      <c r="G31" t="s">
-        <v>2</v>
-      </c>
-      <c r="H31" t="s">
-        <v>2</v>
-      </c>
-      <c r="I31" t="s">
-        <v>2</v>
-      </c>
-      <c r="J31" t="s">
-        <v>2</v>
-      </c>
-      <c r="K31" t="s">
-        <v>2</v>
-      </c>
-      <c r="L31" t="s">
-        <v>2</v>
-      </c>
-      <c r="M31" t="s">
-        <v>2</v>
       </c>
       <c r="N31" t="s">
         <v>791</v>
       </c>
       <c r="O31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>921</v>
+      </c>
+      <c r="B32" t="s">
+        <v>922</v>
+      </c>
+      <c r="C32" t="s">
+        <v>923</v>
+      </c>
+      <c r="D32" t="s">
+        <v>924</v>
+      </c>
+      <c r="E32" t="s">
+        <v>2</v>
+      </c>
+      <c r="F32" t="s">
+        <v>2</v>
+      </c>
+      <c r="G32" t="s">
+        <v>2</v>
+      </c>
+      <c r="H32" t="s">
+        <v>2</v>
+      </c>
+      <c r="I32" t="s">
+        <v>2</v>
+      </c>
+      <c r="J32" t="s">
+        <v>2</v>
+      </c>
+      <c r="K32" t="s">
+        <v>2</v>
+      </c>
+      <c r="L32" t="s">
+        <v>2</v>
+      </c>
+      <c r="M32" t="s">
+        <v>2</v>
+      </c>
+      <c r="N32" t="s">
+        <v>791</v>
+      </c>
+      <c r="O32" t="s">
         <v>29</v>
       </c>
     </row>
@@ -27890,7 +27949,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -27917,7 +27976,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -27994,22 +28053,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>279</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>280</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>281</v>
       </c>
       <c r="D5" t="s">
-        <v>70</v>
+        <v>282</v>
       </c>
       <c r="E5" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F5">
-        <v>25.8</v>
+        <v>24.8</v>
       </c>
       <c r="G5" t="s">
         <v>30</v>
@@ -28017,22 +28076,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>279</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>280</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>281</v>
+        <v>53</v>
       </c>
       <c r="D6" t="s">
-        <v>282</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F6">
-        <v>24.8</v>
+        <v>22.4</v>
       </c>
       <c r="G6" t="s">
         <v>30</v>
@@ -28040,22 +28099,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="B7" t="s">
         <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="E7" t="s">
         <v>37</v>
       </c>
       <c r="F7">
-        <v>22.4</v>
+        <v>21.8</v>
       </c>
       <c r="G7" t="s">
         <v>30</v>
@@ -28063,22 +28122,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B8" t="s">
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E8" t="s">
         <v>37</v>
       </c>
       <c r="F8">
-        <v>21.8</v>
+        <v>19.8</v>
       </c>
       <c r="G8" t="s">
         <v>30</v>
@@ -28086,22 +28145,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="B9" t="s">
         <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>65</v>
       </c>
       <c r="E9" t="s">
         <v>37</v>
       </c>
       <c r="F9">
-        <v>19.8</v>
+        <v>18.6</v>
       </c>
       <c r="G9" t="s">
         <v>30</v>
@@ -28109,22 +28168,22 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="B10" t="s">
         <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="E10" t="s">
         <v>37</v>
       </c>
       <c r="F10">
-        <v>18.6</v>
+        <v>17.8</v>
       </c>
       <c r="G10" t="s">
         <v>30</v>
@@ -28132,22 +28191,22 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="B11" t="s">
         <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="D11" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="E11" t="s">
         <v>37</v>
       </c>
       <c r="F11">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="G11" t="s">
         <v>30</v>
@@ -28155,22 +28214,22 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="D12" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="E12" t="s">
         <v>37</v>
       </c>
       <c r="F12">
-        <v>17.4</v>
+        <v>16</v>
       </c>
       <c r="G12" t="s">
         <v>30</v>
@@ -28178,16 +28237,16 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="E13" t="s">
         <v>37</v>
@@ -28201,16 +28260,16 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="D14" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="E14" t="s">
         <v>37</v>
@@ -28224,22 +28283,22 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="D15" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
       </c>
       <c r="F15">
-        <v>16</v>
+        <v>13.9</v>
       </c>
       <c r="G15" t="s">
         <v>30</v>
@@ -28247,16 +28306,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="B16" t="s">
         <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
       <c r="D16" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
@@ -28270,16 +28329,16 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D17" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E17" t="s">
         <v>37</v>
@@ -28293,16 +28352,16 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B18" t="s">
         <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D18" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E18" t="s">
         <v>37</v>
@@ -28316,22 +28375,22 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D19" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E19" t="s">
         <v>37</v>
       </c>
       <c r="F19">
-        <v>13.9</v>
+        <v>13.3</v>
       </c>
       <c r="G19" t="s">
         <v>30</v>
@@ -28339,22 +28398,22 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="B20" t="s">
         <v>32</v>
       </c>
       <c r="C20" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="D20" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="E20" t="s">
         <v>37</v>
       </c>
       <c r="F20">
-        <v>13.3</v>
+        <v>12.3</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -28362,22 +28421,22 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="B21" t="s">
         <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="D21" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="E21" t="s">
         <v>37</v>
       </c>
       <c r="F21">
-        <v>12.3</v>
+        <v>10.3</v>
       </c>
       <c r="G21" t="s">
         <v>30</v>
@@ -28385,22 +28444,22 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>154</v>
+        <v>273</v>
       </c>
       <c r="B22" t="s">
-        <v>32</v>
+        <v>274</v>
       </c>
       <c r="C22" t="s">
-        <v>155</v>
+        <v>275</v>
       </c>
       <c r="D22" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="E22" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F22">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="G22" t="s">
         <v>30</v>
@@ -28408,16 +28467,16 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="B23" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="C23" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="D23" t="s">
-        <v>143</v>
+        <v>286</v>
       </c>
       <c r="E23" t="s">
         <v>184</v>
@@ -28431,22 +28490,22 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="B24" t="s">
-        <v>284</v>
+        <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>285</v>
+        <v>159</v>
       </c>
       <c r="D24" t="s">
-        <v>286</v>
+        <v>161</v>
       </c>
       <c r="E24" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F24">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G24" t="s">
         <v>30</v>
@@ -28454,22 +28513,22 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>181</v>
       </c>
       <c r="C25" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="D25" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="E25" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F25">
-        <v>9</v>
+        <v>8.3</v>
       </c>
       <c r="G25" t="s">
         <v>30</v>
@@ -28477,22 +28536,22 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>180</v>
+        <v>267</v>
       </c>
       <c r="B26" t="s">
-        <v>181</v>
+        <v>268</v>
       </c>
       <c r="C26" t="s">
-        <v>182</v>
+        <v>269</v>
       </c>
       <c r="D26" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="E26" t="s">
         <v>184</v>
       </c>
       <c r="F26">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G26" t="s">
         <v>30</v>
@@ -28500,16 +28559,16 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B27" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C27" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D27" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="E27" t="s">
         <v>184</v>
@@ -28523,47 +28582,24 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B28" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="C28" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D28" t="s">
-        <v>247</v>
+        <v>2</v>
       </c>
       <c r="E28" t="s">
         <v>184</v>
       </c>
       <c r="F28">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="G28" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>276</v>
-      </c>
-      <c r="B29" t="s">
-        <v>277</v>
-      </c>
-      <c r="C29" t="s">
-        <v>278</v>
-      </c>
-      <c r="D29" t="s">
-        <v>2</v>
-      </c>
-      <c r="E29" t="s">
-        <v>184</v>
-      </c>
-      <c r="F29">
-        <v>0.8</v>
-      </c>
-      <c r="G29" t="s">
         <v>30</v>
       </c>
     </row>
@@ -28614,27 +28650,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lessons: add and publish Gimel (letter 3)
Normalizes the Gimel source lesson, removes its vowel-length claims per
the course editorial rules, holds out the one MATCH_PAIRS exercise whose
length claim lives in unoverridable pairs data, flags unintroduced-letter
distractors, and publishes with SEO title/meta/H1 and a guide link.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,12 +17,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8084" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8093" uniqueCount="935">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
   <si>
-    <t>Generated: 2026-10-14 by scripts/seo/build-core.mjs (npm run seo:build)</t>
+    <t>Generated: 2026-10-15 by scripts/seo/build-core.mjs (npm run seo:build)</t>
   </si>
   <si>
     <t/>
@@ -2690,6 +2690,18 @@
   </si>
   <si>
     <t>vet hebrew letter; hebrew bet pronunciation; hebrew letter bet sound; learn hebrew letter bet; bet hebrew letter exercises; bet with dagesh</t>
+  </si>
+  <si>
+    <t>Gimel Hebrew Letter (ג): Sound &amp; Words</t>
+  </si>
+  <si>
+    <t>Gimel Hebrew Letter (ג): Sound, Words &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Gimel (ג): its [g] sound, with example words like גַג (roof) and אַגַב (incidentally), plus interactive practice.</t>
+  </si>
+  <si>
+    <t>hebrew gimel pronunciation; hebrew letter gimel sound; learn hebrew letter gimel; gimel hebrew letter exercises; gimmel hebrew letter; how to recognize gimel</t>
   </si>
   <si>
     <t>Hebrew Phrases for Beginners: 30 Useful Phrases | HebrewEdu</t>
@@ -3895,7 +3907,7 @@
         <v>115</v>
       </c>
       <c r="G21" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H21" t="s">
         <v>30</v>
@@ -14646,7 +14658,7 @@
         <v>306</v>
       </c>
       <c r="L155" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M155" t="s">
         <v>30</v>
@@ -14705,7 +14717,7 @@
         <v>306</v>
       </c>
       <c r="L156" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M156" t="s">
         <v>312</v>
@@ -14764,7 +14776,7 @@
         <v>306</v>
       </c>
       <c r="L157" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M157" t="s">
         <v>312</v>
@@ -14823,7 +14835,7 @@
         <v>306</v>
       </c>
       <c r="L158" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M158" t="s">
         <v>312</v>
@@ -14882,7 +14894,7 @@
         <v>306</v>
       </c>
       <c r="L159" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M159" t="s">
         <v>312</v>
@@ -14941,7 +14953,7 @@
         <v>306</v>
       </c>
       <c r="L160" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M160" t="s">
         <v>312</v>
@@ -15000,7 +15012,7 @@
         <v>306</v>
       </c>
       <c r="L161" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M161" t="s">
         <v>312</v>
@@ -26420,7 +26432,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -27566,7 +27578,7 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>282</v>
+        <v>115</v>
       </c>
       <c r="B25" t="s">
         <v>891</v>
@@ -27578,10 +27590,10 @@
         <v>893</v>
       </c>
       <c r="E25" t="s">
-        <v>279</v>
+        <v>112</v>
       </c>
       <c r="F25" t="s">
-        <v>755</v>
+        <v>113</v>
       </c>
       <c r="G25" t="s">
         <v>894</v>
@@ -27613,7 +27625,7 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>203</v>
+        <v>282</v>
       </c>
       <c r="B26" t="s">
         <v>895</v>
@@ -27625,10 +27637,10 @@
         <v>897</v>
       </c>
       <c r="E26" t="s">
-        <v>201</v>
+        <v>279</v>
       </c>
       <c r="F26" t="s">
-        <v>202</v>
+        <v>755</v>
       </c>
       <c r="G26" t="s">
         <v>898</v>
@@ -27652,7 +27664,7 @@
         <v>2</v>
       </c>
       <c r="N26" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O26" t="s">
         <v>29</v>
@@ -27660,7 +27672,7 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>171</v>
+        <v>203</v>
       </c>
       <c r="B27" t="s">
         <v>899</v>
@@ -27672,10 +27684,10 @@
         <v>901</v>
       </c>
       <c r="E27" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="F27" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="G27" t="s">
         <v>902</v>
@@ -27707,7 +27719,7 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>228</v>
+        <v>171</v>
       </c>
       <c r="B28" t="s">
         <v>903</v>
@@ -27719,10 +27731,10 @@
         <v>905</v>
       </c>
       <c r="E28" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="F28" t="s">
-        <v>257</v>
+        <v>169</v>
       </c>
       <c r="G28" t="s">
         <v>906</v>
@@ -27754,7 +27766,7 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>286</v>
+        <v>228</v>
       </c>
       <c r="B29" t="s">
         <v>907</v>
@@ -27766,10 +27778,10 @@
         <v>909</v>
       </c>
       <c r="E29" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F29" t="s">
-        <v>763</v>
+        <v>257</v>
       </c>
       <c r="G29" t="s">
         <v>910</v>
@@ -27793,7 +27805,7 @@
         <v>2</v>
       </c>
       <c r="N29" t="s">
-        <v>882</v>
+        <v>791</v>
       </c>
       <c r="O29" t="s">
         <v>29</v>
@@ -27801,46 +27813,46 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>286</v>
+      </c>
+      <c r="B30" t="s">
         <v>911</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>912</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>913</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
+        <v>283</v>
+      </c>
+      <c r="F30" t="s">
+        <v>763</v>
+      </c>
+      <c r="G30" t="s">
         <v>914</v>
       </c>
-      <c r="E30" t="s">
-        <v>2</v>
-      </c>
-      <c r="F30" t="s">
-        <v>2</v>
-      </c>
-      <c r="G30" t="s">
-        <v>2</v>
-      </c>
       <c r="H30" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I30" t="s">
-        <v>492</v>
+        <v>2</v>
       </c>
       <c r="J30" t="s">
-        <v>915</v>
+        <v>2</v>
       </c>
       <c r="K30" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="L30" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="M30" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N30" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O30" t="s">
         <v>29</v>
@@ -27848,16 +27860,16 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>915</v>
+      </c>
+      <c r="B31" t="s">
         <v>916</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>917</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>918</v>
-      </c>
-      <c r="D31" t="s">
-        <v>919</v>
       </c>
       <c r="E31" t="s">
         <v>2</v>
@@ -27872,19 +27884,19 @@
         <v>80</v>
       </c>
       <c r="I31" t="s">
-        <v>415</v>
+        <v>492</v>
       </c>
       <c r="J31" t="s">
-        <v>353</v>
+        <v>919</v>
       </c>
       <c r="K31" t="s">
         <v>80</v>
       </c>
       <c r="L31" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M31" t="s">
-        <v>920</v>
+        <v>64</v>
       </c>
       <c r="N31" t="s">
         <v>791</v>
@@ -27895,48 +27907,95 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>920</v>
+      </c>
+      <c r="B32" t="s">
         <v>921</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>922</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>923</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
+        <v>2</v>
+      </c>
+      <c r="F32" t="s">
+        <v>2</v>
+      </c>
+      <c r="G32" t="s">
+        <v>2</v>
+      </c>
+      <c r="H32" t="s">
+        <v>80</v>
+      </c>
+      <c r="I32" t="s">
+        <v>415</v>
+      </c>
+      <c r="J32" t="s">
+        <v>353</v>
+      </c>
+      <c r="K32" t="s">
+        <v>80</v>
+      </c>
+      <c r="L32" t="s">
+        <v>95</v>
+      </c>
+      <c r="M32" t="s">
         <v>924</v>
-      </c>
-      <c r="E32" t="s">
-        <v>2</v>
-      </c>
-      <c r="F32" t="s">
-        <v>2</v>
-      </c>
-      <c r="G32" t="s">
-        <v>2</v>
-      </c>
-      <c r="H32" t="s">
-        <v>2</v>
-      </c>
-      <c r="I32" t="s">
-        <v>2</v>
-      </c>
-      <c r="J32" t="s">
-        <v>2</v>
-      </c>
-      <c r="K32" t="s">
-        <v>2</v>
-      </c>
-      <c r="L32" t="s">
-        <v>2</v>
-      </c>
-      <c r="M32" t="s">
-        <v>2</v>
       </c>
       <c r="N32" t="s">
         <v>791</v>
       </c>
       <c r="O32" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>925</v>
+      </c>
+      <c r="B33" t="s">
+        <v>926</v>
+      </c>
+      <c r="C33" t="s">
+        <v>927</v>
+      </c>
+      <c r="D33" t="s">
+        <v>928</v>
+      </c>
+      <c r="E33" t="s">
+        <v>2</v>
+      </c>
+      <c r="F33" t="s">
+        <v>2</v>
+      </c>
+      <c r="G33" t="s">
+        <v>2</v>
+      </c>
+      <c r="H33" t="s">
+        <v>2</v>
+      </c>
+      <c r="I33" t="s">
+        <v>2</v>
+      </c>
+      <c r="J33" t="s">
+        <v>2</v>
+      </c>
+      <c r="K33" t="s">
+        <v>2</v>
+      </c>
+      <c r="L33" t="s">
+        <v>2</v>
+      </c>
+      <c r="M33" t="s">
+        <v>2</v>
+      </c>
+      <c r="N33" t="s">
+        <v>791</v>
+      </c>
+      <c r="O33" t="s">
         <v>29</v>
       </c>
     </row>
@@ -27949,7 +28008,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -27976,7 +28035,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -28283,16 +28342,16 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
       <c r="D15" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
@@ -28306,16 +28365,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B16" t="s">
         <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D16" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
@@ -28329,16 +28388,16 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D17" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E17" t="s">
         <v>37</v>
@@ -28352,22 +28411,22 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
         <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D18" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E18" t="s">
         <v>37</v>
       </c>
       <c r="F18">
-        <v>13.9</v>
+        <v>13.3</v>
       </c>
       <c r="G18" t="s">
         <v>30</v>
@@ -28375,22 +28434,22 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="D19" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="E19" t="s">
         <v>37</v>
       </c>
       <c r="F19">
-        <v>13.3</v>
+        <v>12.3</v>
       </c>
       <c r="G19" t="s">
         <v>30</v>
@@ -28398,22 +28457,22 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="B20" t="s">
         <v>32</v>
       </c>
       <c r="C20" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="D20" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="E20" t="s">
         <v>37</v>
       </c>
       <c r="F20">
-        <v>12.3</v>
+        <v>10.3</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -28421,22 +28480,22 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>154</v>
+        <v>273</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>274</v>
       </c>
       <c r="C21" t="s">
-        <v>155</v>
+        <v>275</v>
       </c>
       <c r="D21" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="E21" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F21">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="G21" t="s">
         <v>30</v>
@@ -28444,16 +28503,16 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="B22" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="C22" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="D22" t="s">
-        <v>143</v>
+        <v>286</v>
       </c>
       <c r="E22" t="s">
         <v>184</v>
@@ -28467,22 +28526,22 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="B23" t="s">
-        <v>284</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>285</v>
+        <v>159</v>
       </c>
       <c r="D23" t="s">
-        <v>286</v>
+        <v>161</v>
       </c>
       <c r="E23" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G23" t="s">
         <v>30</v>
@@ -28490,22 +28549,22 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>181</v>
       </c>
       <c r="C24" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="D24" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="E24" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F24">
-        <v>9</v>
+        <v>8.3</v>
       </c>
       <c r="G24" t="s">
         <v>30</v>
@@ -28513,22 +28572,22 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>180</v>
+        <v>267</v>
       </c>
       <c r="B25" t="s">
-        <v>181</v>
+        <v>268</v>
       </c>
       <c r="C25" t="s">
-        <v>182</v>
+        <v>269</v>
       </c>
       <c r="D25" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="E25" t="s">
         <v>184</v>
       </c>
       <c r="F25">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G25" t="s">
         <v>30</v>
@@ -28536,16 +28595,16 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B26" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C26" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D26" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="E26" t="s">
         <v>184</v>
@@ -28559,47 +28618,24 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B27" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="C27" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D27" t="s">
-        <v>247</v>
+        <v>2</v>
       </c>
       <c r="E27" t="s">
         <v>184</v>
       </c>
       <c r="F27">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="G27" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>276</v>
-      </c>
-      <c r="B28" t="s">
-        <v>277</v>
-      </c>
-      <c r="C28" t="s">
-        <v>278</v>
-      </c>
-      <c r="D28" t="s">
-        <v>2</v>
-      </c>
-      <c r="E28" t="s">
-        <v>184</v>
-      </c>
-      <c r="F28">
-        <v>0.8</v>
-      </c>
-      <c r="G28" t="s">
         <v>30</v>
       </c>
     </row>
@@ -28650,27 +28686,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lessons: add and publish Dalet (letter 4)
Editorial fixes: removed vowel-length "short [a]" claims from four
exercise tips (Patah is [a] in Modern Hebrew); flagged unintroduced-letter
distractors (optional, matches Aleph/Bet/Gimel precedent). Registered in
the SEO core (pages.csv/keywords.csv/clusters.csv) and linked from the
alphabet guide.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8093" uniqueCount="935">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8102" uniqueCount="939">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
@@ -2702,6 +2702,18 @@
   </si>
   <si>
     <t>hebrew gimel pronunciation; hebrew letter gimel sound; learn hebrew letter gimel; gimel hebrew letter exercises; gimmel hebrew letter; how to recognize gimel</t>
+  </si>
+  <si>
+    <t>Dalet Hebrew Letter (ד): Sound &amp; Words</t>
+  </si>
+  <si>
+    <t>Dalet Hebrew Letter (ד): Sound, Words &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Dalet (ד): its [d] sound, with example words like דַג (fish) and אָבַד (lost), plus interactive practice.</t>
+  </si>
+  <si>
+    <t>hebrew dalet pronunciation; hebrew letter dalet sound; learn hebrew letter dalet; dalet hebrew letter exercises; daleth hebrew letter; dalet vs resh hebrew letters</t>
   </si>
   <si>
     <t>Hebrew Phrases for Beginners: 30 Useful Phrases | HebrewEdu</t>
@@ -4052,7 +4064,7 @@
         <v>133</v>
       </c>
       <c r="G26" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H26" t="s">
         <v>30</v>
@@ -15071,7 +15083,7 @@
         <v>306</v>
       </c>
       <c r="L162" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M162" t="s">
         <v>30</v>
@@ -15130,7 +15142,7 @@
         <v>306</v>
       </c>
       <c r="L163" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M163" t="s">
         <v>312</v>
@@ -15189,7 +15201,7 @@
         <v>306</v>
       </c>
       <c r="L164" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M164" t="s">
         <v>312</v>
@@ -15248,7 +15260,7 @@
         <v>306</v>
       </c>
       <c r="L165" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M165" t="s">
         <v>312</v>
@@ -15307,7 +15319,7 @@
         <v>306</v>
       </c>
       <c r="L166" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M166" t="s">
         <v>312</v>
@@ -15366,7 +15378,7 @@
         <v>306</v>
       </c>
       <c r="L167" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M167" t="s">
         <v>312</v>
@@ -15425,7 +15437,7 @@
         <v>306</v>
       </c>
       <c r="L168" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M168" t="s">
         <v>312</v>
@@ -26432,7 +26444,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -27625,7 +27637,7 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>282</v>
+        <v>133</v>
       </c>
       <c r="B26" t="s">
         <v>895</v>
@@ -27637,10 +27649,10 @@
         <v>897</v>
       </c>
       <c r="E26" t="s">
-        <v>279</v>
+        <v>131</v>
       </c>
       <c r="F26" t="s">
-        <v>755</v>
+        <v>132</v>
       </c>
       <c r="G26" t="s">
         <v>898</v>
@@ -27672,7 +27684,7 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>203</v>
+        <v>282</v>
       </c>
       <c r="B27" t="s">
         <v>899</v>
@@ -27684,10 +27696,10 @@
         <v>901</v>
       </c>
       <c r="E27" t="s">
-        <v>201</v>
+        <v>279</v>
       </c>
       <c r="F27" t="s">
-        <v>202</v>
+        <v>755</v>
       </c>
       <c r="G27" t="s">
         <v>902</v>
@@ -27711,7 +27723,7 @@
         <v>2</v>
       </c>
       <c r="N27" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O27" t="s">
         <v>29</v>
@@ -27719,7 +27731,7 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>171</v>
+        <v>203</v>
       </c>
       <c r="B28" t="s">
         <v>903</v>
@@ -27731,10 +27743,10 @@
         <v>905</v>
       </c>
       <c r="E28" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="F28" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="G28" t="s">
         <v>906</v>
@@ -27766,7 +27778,7 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>228</v>
+        <v>171</v>
       </c>
       <c r="B29" t="s">
         <v>907</v>
@@ -27778,10 +27790,10 @@
         <v>909</v>
       </c>
       <c r="E29" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="F29" t="s">
-        <v>257</v>
+        <v>169</v>
       </c>
       <c r="G29" t="s">
         <v>910</v>
@@ -27813,7 +27825,7 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>286</v>
+        <v>228</v>
       </c>
       <c r="B30" t="s">
         <v>911</v>
@@ -27825,10 +27837,10 @@
         <v>913</v>
       </c>
       <c r="E30" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F30" t="s">
-        <v>763</v>
+        <v>257</v>
       </c>
       <c r="G30" t="s">
         <v>914</v>
@@ -27852,7 +27864,7 @@
         <v>2</v>
       </c>
       <c r="N30" t="s">
-        <v>882</v>
+        <v>791</v>
       </c>
       <c r="O30" t="s">
         <v>29</v>
@@ -27860,46 +27872,46 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>286</v>
+      </c>
+      <c r="B31" t="s">
         <v>915</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>916</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>917</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
+        <v>283</v>
+      </c>
+      <c r="F31" t="s">
+        <v>763</v>
+      </c>
+      <c r="G31" t="s">
         <v>918</v>
       </c>
-      <c r="E31" t="s">
-        <v>2</v>
-      </c>
-      <c r="F31" t="s">
-        <v>2</v>
-      </c>
-      <c r="G31" t="s">
-        <v>2</v>
-      </c>
       <c r="H31" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I31" t="s">
-        <v>492</v>
+        <v>2</v>
       </c>
       <c r="J31" t="s">
-        <v>919</v>
+        <v>2</v>
       </c>
       <c r="K31" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="L31" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="M31" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N31" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O31" t="s">
         <v>29</v>
@@ -27907,16 +27919,16 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>919</v>
+      </c>
+      <c r="B32" t="s">
         <v>920</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>921</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>922</v>
-      </c>
-      <c r="D32" t="s">
-        <v>923</v>
       </c>
       <c r="E32" t="s">
         <v>2</v>
@@ -27931,19 +27943,19 @@
         <v>80</v>
       </c>
       <c r="I32" t="s">
-        <v>415</v>
+        <v>492</v>
       </c>
       <c r="J32" t="s">
-        <v>353</v>
+        <v>923</v>
       </c>
       <c r="K32" t="s">
         <v>80</v>
       </c>
       <c r="L32" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M32" t="s">
-        <v>924</v>
+        <v>64</v>
       </c>
       <c r="N32" t="s">
         <v>791</v>
@@ -27954,48 +27966,95 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>924</v>
+      </c>
+      <c r="B33" t="s">
         <v>925</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>926</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>927</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
+        <v>2</v>
+      </c>
+      <c r="F33" t="s">
+        <v>2</v>
+      </c>
+      <c r="G33" t="s">
+        <v>2</v>
+      </c>
+      <c r="H33" t="s">
+        <v>80</v>
+      </c>
+      <c r="I33" t="s">
+        <v>415</v>
+      </c>
+      <c r="J33" t="s">
+        <v>353</v>
+      </c>
+      <c r="K33" t="s">
+        <v>80</v>
+      </c>
+      <c r="L33" t="s">
+        <v>95</v>
+      </c>
+      <c r="M33" t="s">
         <v>928</v>
-      </c>
-      <c r="E33" t="s">
-        <v>2</v>
-      </c>
-      <c r="F33" t="s">
-        <v>2</v>
-      </c>
-      <c r="G33" t="s">
-        <v>2</v>
-      </c>
-      <c r="H33" t="s">
-        <v>2</v>
-      </c>
-      <c r="I33" t="s">
-        <v>2</v>
-      </c>
-      <c r="J33" t="s">
-        <v>2</v>
-      </c>
-      <c r="K33" t="s">
-        <v>2</v>
-      </c>
-      <c r="L33" t="s">
-        <v>2</v>
-      </c>
-      <c r="M33" t="s">
-        <v>2</v>
       </c>
       <c r="N33" t="s">
         <v>791</v>
       </c>
       <c r="O33" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>929</v>
+      </c>
+      <c r="B34" t="s">
+        <v>930</v>
+      </c>
+      <c r="C34" t="s">
+        <v>931</v>
+      </c>
+      <c r="D34" t="s">
+        <v>932</v>
+      </c>
+      <c r="E34" t="s">
+        <v>2</v>
+      </c>
+      <c r="F34" t="s">
+        <v>2</v>
+      </c>
+      <c r="G34" t="s">
+        <v>2</v>
+      </c>
+      <c r="H34" t="s">
+        <v>2</v>
+      </c>
+      <c r="I34" t="s">
+        <v>2</v>
+      </c>
+      <c r="J34" t="s">
+        <v>2</v>
+      </c>
+      <c r="K34" t="s">
+        <v>2</v>
+      </c>
+      <c r="L34" t="s">
+        <v>2</v>
+      </c>
+      <c r="M34" t="s">
+        <v>2</v>
+      </c>
+      <c r="N34" t="s">
+        <v>791</v>
+      </c>
+      <c r="O34" t="s">
         <v>29</v>
       </c>
     </row>
@@ -28008,7 +28067,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -28035,7 +28094,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -28319,22 +28378,22 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D14" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E14" t="s">
         <v>37</v>
       </c>
       <c r="F14">
-        <v>16</v>
+        <v>13.9</v>
       </c>
       <c r="G14" t="s">
         <v>30</v>
@@ -28342,16 +28401,16 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D15" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
@@ -28365,16 +28424,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B16" t="s">
         <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D16" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
@@ -28388,22 +28447,22 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D17" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E17" t="s">
         <v>37</v>
       </c>
       <c r="F17">
-        <v>13.9</v>
+        <v>13.3</v>
       </c>
       <c r="G17" t="s">
         <v>30</v>
@@ -28411,22 +28470,22 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="B18" t="s">
         <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="D18" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="E18" t="s">
         <v>37</v>
       </c>
       <c r="F18">
-        <v>13.3</v>
+        <v>12.3</v>
       </c>
       <c r="G18" t="s">
         <v>30</v>
@@ -28434,22 +28493,22 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="D19" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="E19" t="s">
         <v>37</v>
       </c>
       <c r="F19">
-        <v>12.3</v>
+        <v>10.3</v>
       </c>
       <c r="G19" t="s">
         <v>30</v>
@@ -28457,22 +28516,22 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>154</v>
+        <v>273</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>274</v>
       </c>
       <c r="C20" t="s">
-        <v>155</v>
+        <v>275</v>
       </c>
       <c r="D20" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="E20" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F20">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -28480,16 +28539,16 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="B21" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="C21" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="D21" t="s">
-        <v>143</v>
+        <v>286</v>
       </c>
       <c r="E21" t="s">
         <v>184</v>
@@ -28503,22 +28562,22 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="B22" t="s">
-        <v>284</v>
+        <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>285</v>
+        <v>159</v>
       </c>
       <c r="D22" t="s">
-        <v>286</v>
+        <v>161</v>
       </c>
       <c r="E22" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F22">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G22" t="s">
         <v>30</v>
@@ -28526,22 +28585,22 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>181</v>
       </c>
       <c r="C23" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="D23" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="E23" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F23">
-        <v>9</v>
+        <v>8.3</v>
       </c>
       <c r="G23" t="s">
         <v>30</v>
@@ -28549,22 +28608,22 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>180</v>
+        <v>267</v>
       </c>
       <c r="B24" t="s">
-        <v>181</v>
+        <v>268</v>
       </c>
       <c r="C24" t="s">
-        <v>182</v>
+        <v>269</v>
       </c>
       <c r="D24" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="E24" t="s">
         <v>184</v>
       </c>
       <c r="F24">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G24" t="s">
         <v>30</v>
@@ -28572,16 +28631,16 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B25" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C25" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D25" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="E25" t="s">
         <v>184</v>
@@ -28595,47 +28654,24 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B26" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="C26" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D26" t="s">
-        <v>247</v>
+        <v>2</v>
       </c>
       <c r="E26" t="s">
         <v>184</v>
       </c>
       <c r="F26">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="G26" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>276</v>
-      </c>
-      <c r="B27" t="s">
-        <v>277</v>
-      </c>
-      <c r="C27" t="s">
-        <v>278</v>
-      </c>
-      <c r="D27" t="s">
-        <v>2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>184</v>
-      </c>
-      <c r="F27">
-        <v>0.8</v>
-      </c>
-      <c r="G27" t="s">
         <v>30</v>
       </c>
     </row>
@@ -28686,27 +28722,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lessons: prepare He (letter 5), preview-only pending weekly limit
Editorial fixes: removed three vowel-length claims; flagged two
unintroduced-letter distractors; held out two empty TITLE_IMAGE blocks
(also empty in Vav/Pe/Tsadi's unpublished sources — recommend a follow-up
task). Registered in the SEO core as "planned" (publish deferred: Bet,
Gimel and Dalet already fill this ISO week's 3-lesson limit). Owner has
approved publishing once the next allowed date (2026-10-19) arrives.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8102" uniqueCount="939">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8117" uniqueCount="943">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
@@ -2714,6 +2714,18 @@
   </si>
   <si>
     <t>hebrew dalet pronunciation; hebrew letter dalet sound; learn hebrew letter dalet; dalet hebrew letter exercises; daleth hebrew letter; dalet vs resh hebrew letters</t>
+  </si>
+  <si>
+    <t>Hey Hebrew Letter (ה): Sound &amp; Vowels</t>
+  </si>
+  <si>
+    <t>Hey Hebrew Letter (ה): Sound, Vowels &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Hey (ה): its soft [h] sound, the Tsere and Segol [e] vowels, and example words like הֶגֶה (steering wheel), plus practice.</t>
+  </si>
+  <si>
+    <t>he hebrew letter; hebrew he pronunciation; hebrew letter he sound; learn hebrew letter he; he hebrew letter exercises; he vs chet hebrew letters; he at end of hebrew word</t>
   </si>
   <si>
     <t>Hebrew Phrases for Beginners: 30 Useful Phrases | HebrewEdu</t>
@@ -26444,7 +26456,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -27684,7 +27696,7 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>282</v>
+        <v>111</v>
       </c>
       <c r="B27" t="s">
         <v>899</v>
@@ -27696,10 +27708,10 @@
         <v>901</v>
       </c>
       <c r="E27" t="s">
-        <v>279</v>
+        <v>109</v>
       </c>
       <c r="F27" t="s">
-        <v>755</v>
+        <v>110</v>
       </c>
       <c r="G27" t="s">
         <v>902</v>
@@ -27726,12 +27738,12 @@
         <v>882</v>
       </c>
       <c r="O27" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>203</v>
+        <v>282</v>
       </c>
       <c r="B28" t="s">
         <v>903</v>
@@ -27743,10 +27755,10 @@
         <v>905</v>
       </c>
       <c r="E28" t="s">
-        <v>201</v>
+        <v>279</v>
       </c>
       <c r="F28" t="s">
-        <v>202</v>
+        <v>755</v>
       </c>
       <c r="G28" t="s">
         <v>906</v>
@@ -27770,7 +27782,7 @@
         <v>2</v>
       </c>
       <c r="N28" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O28" t="s">
         <v>29</v>
@@ -27778,7 +27790,7 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>171</v>
+        <v>203</v>
       </c>
       <c r="B29" t="s">
         <v>907</v>
@@ -27790,10 +27802,10 @@
         <v>909</v>
       </c>
       <c r="E29" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="F29" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="G29" t="s">
         <v>910</v>
@@ -27825,7 +27837,7 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>228</v>
+        <v>171</v>
       </c>
       <c r="B30" t="s">
         <v>911</v>
@@ -27837,10 +27849,10 @@
         <v>913</v>
       </c>
       <c r="E30" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="F30" t="s">
-        <v>257</v>
+        <v>169</v>
       </c>
       <c r="G30" t="s">
         <v>914</v>
@@ -27872,7 +27884,7 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>286</v>
+        <v>228</v>
       </c>
       <c r="B31" t="s">
         <v>915</v>
@@ -27884,10 +27896,10 @@
         <v>917</v>
       </c>
       <c r="E31" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F31" t="s">
-        <v>763</v>
+        <v>257</v>
       </c>
       <c r="G31" t="s">
         <v>918</v>
@@ -27911,7 +27923,7 @@
         <v>2</v>
       </c>
       <c r="N31" t="s">
-        <v>882</v>
+        <v>791</v>
       </c>
       <c r="O31" t="s">
         <v>29</v>
@@ -27919,46 +27931,46 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>286</v>
+      </c>
+      <c r="B32" t="s">
         <v>919</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>920</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>921</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
+        <v>283</v>
+      </c>
+      <c r="F32" t="s">
+        <v>763</v>
+      </c>
+      <c r="G32" t="s">
         <v>922</v>
       </c>
-      <c r="E32" t="s">
-        <v>2</v>
-      </c>
-      <c r="F32" t="s">
-        <v>2</v>
-      </c>
-      <c r="G32" t="s">
-        <v>2</v>
-      </c>
       <c r="H32" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I32" t="s">
-        <v>492</v>
+        <v>2</v>
       </c>
       <c r="J32" t="s">
-        <v>923</v>
+        <v>2</v>
       </c>
       <c r="K32" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="L32" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="M32" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N32" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O32" t="s">
         <v>29</v>
@@ -27966,16 +27978,16 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>923</v>
+      </c>
+      <c r="B33" t="s">
         <v>924</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>925</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>926</v>
-      </c>
-      <c r="D33" t="s">
-        <v>927</v>
       </c>
       <c r="E33" t="s">
         <v>2</v>
@@ -27990,19 +28002,19 @@
         <v>80</v>
       </c>
       <c r="I33" t="s">
-        <v>415</v>
+        <v>492</v>
       </c>
       <c r="J33" t="s">
-        <v>353</v>
+        <v>927</v>
       </c>
       <c r="K33" t="s">
         <v>80</v>
       </c>
       <c r="L33" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M33" t="s">
-        <v>928</v>
+        <v>64</v>
       </c>
       <c r="N33" t="s">
         <v>791</v>
@@ -28013,48 +28025,95 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>928</v>
+      </c>
+      <c r="B34" t="s">
         <v>929</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>930</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>931</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
+        <v>2</v>
+      </c>
+      <c r="F34" t="s">
+        <v>2</v>
+      </c>
+      <c r="G34" t="s">
+        <v>2</v>
+      </c>
+      <c r="H34" t="s">
+        <v>80</v>
+      </c>
+      <c r="I34" t="s">
+        <v>415</v>
+      </c>
+      <c r="J34" t="s">
+        <v>353</v>
+      </c>
+      <c r="K34" t="s">
+        <v>80</v>
+      </c>
+      <c r="L34" t="s">
+        <v>95</v>
+      </c>
+      <c r="M34" t="s">
         <v>932</v>
-      </c>
-      <c r="E34" t="s">
-        <v>2</v>
-      </c>
-      <c r="F34" t="s">
-        <v>2</v>
-      </c>
-      <c r="G34" t="s">
-        <v>2</v>
-      </c>
-      <c r="H34" t="s">
-        <v>2</v>
-      </c>
-      <c r="I34" t="s">
-        <v>2</v>
-      </c>
-      <c r="J34" t="s">
-        <v>2</v>
-      </c>
-      <c r="K34" t="s">
-        <v>2</v>
-      </c>
-      <c r="L34" t="s">
-        <v>2</v>
-      </c>
-      <c r="M34" t="s">
-        <v>2</v>
       </c>
       <c r="N34" t="s">
         <v>791</v>
       </c>
       <c r="O34" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>933</v>
+      </c>
+      <c r="B35" t="s">
+        <v>934</v>
+      </c>
+      <c r="C35" t="s">
+        <v>935</v>
+      </c>
+      <c r="D35" t="s">
+        <v>936</v>
+      </c>
+      <c r="E35" t="s">
+        <v>2</v>
+      </c>
+      <c r="F35" t="s">
+        <v>2</v>
+      </c>
+      <c r="G35" t="s">
+        <v>2</v>
+      </c>
+      <c r="H35" t="s">
+        <v>2</v>
+      </c>
+      <c r="I35" t="s">
+        <v>2</v>
+      </c>
+      <c r="J35" t="s">
+        <v>2</v>
+      </c>
+      <c r="K35" t="s">
+        <v>2</v>
+      </c>
+      <c r="L35" t="s">
+        <v>2</v>
+      </c>
+      <c r="M35" t="s">
+        <v>2</v>
+      </c>
+      <c r="N35" t="s">
+        <v>791</v>
+      </c>
+      <c r="O35" t="s">
         <v>29</v>
       </c>
     </row>
@@ -28094,7 +28153,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -28722,27 +28781,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>935</v>
+        <v>939</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>936</v>
+        <v>940</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>938</v>
+        <v>942</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lessons: publish He (letter 5)
Weekly limit cleared (new ISO week starting 2026-10-19); owner approved.
Flips editorial/publication flags, registers He as published in the SEO
core, links it from the alphabet guide, and updates the hub test's
published-lesson assertions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,12 +17,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8117" uniqueCount="943">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8111" uniqueCount="943">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
   <si>
-    <t>Generated: 2026-10-15 by scripts/seo/build-core.mjs (npm run seo:build)</t>
+    <t>Generated: 2026-10-19 by scripts/seo/build-core.mjs (npm run seo:build)</t>
   </si>
   <si>
     <t/>
@@ -3902,7 +3902,7 @@
         <v>111</v>
       </c>
       <c r="G20" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H20" t="s">
         <v>30</v>
@@ -15508,7 +15508,7 @@
         <v>306</v>
       </c>
       <c r="L169" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M169" t="s">
         <v>30</v>
@@ -15567,7 +15567,7 @@
         <v>306</v>
       </c>
       <c r="L170" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M170" t="s">
         <v>312</v>
@@ -15626,7 +15626,7 @@
         <v>306</v>
       </c>
       <c r="L171" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M171" t="s">
         <v>312</v>
@@ -15685,7 +15685,7 @@
         <v>306</v>
       </c>
       <c r="L172" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M172" t="s">
         <v>312</v>
@@ -15744,7 +15744,7 @@
         <v>306</v>
       </c>
       <c r="L173" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M173" t="s">
         <v>312</v>
@@ -15803,7 +15803,7 @@
         <v>306</v>
       </c>
       <c r="L174" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M174" t="s">
         <v>312</v>
@@ -15862,7 +15862,7 @@
         <v>306</v>
       </c>
       <c r="L175" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M175" t="s">
         <v>312</v>
@@ -15921,7 +15921,7 @@
         <v>306</v>
       </c>
       <c r="L176" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M176" t="s">
         <v>312</v>
@@ -27738,7 +27738,7 @@
         <v>882</v>
       </c>
       <c r="O27" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -28126,7 +28126,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -28414,22 +28414,22 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="D13" t="s">
-        <v>111</v>
+        <v>138</v>
       </c>
       <c r="E13" t="s">
         <v>37</v>
       </c>
       <c r="F13">
-        <v>16</v>
+        <v>13.9</v>
       </c>
       <c r="G13" t="s">
         <v>30</v>
@@ -28437,16 +28437,16 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E14" t="s">
         <v>37</v>
@@ -28460,16 +28460,16 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D15" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
@@ -28483,22 +28483,22 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B16" t="s">
         <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D16" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
       </c>
       <c r="F16">
-        <v>13.9</v>
+        <v>13.3</v>
       </c>
       <c r="G16" t="s">
         <v>30</v>
@@ -28506,22 +28506,22 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="D17" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="E17" t="s">
         <v>37</v>
       </c>
       <c r="F17">
-        <v>13.3</v>
+        <v>12.3</v>
       </c>
       <c r="G17" t="s">
         <v>30</v>
@@ -28529,22 +28529,22 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="B18" t="s">
         <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="D18" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="E18" t="s">
         <v>37</v>
       </c>
       <c r="F18">
-        <v>12.3</v>
+        <v>10.3</v>
       </c>
       <c r="G18" t="s">
         <v>30</v>
@@ -28552,22 +28552,22 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>154</v>
+        <v>273</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>274</v>
       </c>
       <c r="C19" t="s">
-        <v>155</v>
+        <v>275</v>
       </c>
       <c r="D19" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="E19" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F19">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="G19" t="s">
         <v>30</v>
@@ -28575,16 +28575,16 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="B20" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="C20" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="D20" t="s">
-        <v>143</v>
+        <v>286</v>
       </c>
       <c r="E20" t="s">
         <v>184</v>
@@ -28598,22 +28598,22 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="B21" t="s">
-        <v>284</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>285</v>
+        <v>159</v>
       </c>
       <c r="D21" t="s">
-        <v>286</v>
+        <v>161</v>
       </c>
       <c r="E21" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F21">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G21" t="s">
         <v>30</v>
@@ -28621,22 +28621,22 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="B22" t="s">
-        <v>32</v>
+        <v>181</v>
       </c>
       <c r="C22" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="D22" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="E22" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F22">
-        <v>9</v>
+        <v>8.3</v>
       </c>
       <c r="G22" t="s">
         <v>30</v>
@@ -28644,22 +28644,22 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>180</v>
+        <v>267</v>
       </c>
       <c r="B23" t="s">
-        <v>181</v>
+        <v>268</v>
       </c>
       <c r="C23" t="s">
-        <v>182</v>
+        <v>269</v>
       </c>
       <c r="D23" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="E23" t="s">
         <v>184</v>
       </c>
       <c r="F23">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G23" t="s">
         <v>30</v>
@@ -28667,16 +28667,16 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B24" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C24" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D24" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="E24" t="s">
         <v>184</v>
@@ -28690,47 +28690,24 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B25" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="C25" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D25" t="s">
-        <v>247</v>
+        <v>2</v>
       </c>
       <c r="E25" t="s">
         <v>184</v>
       </c>
       <c r="F25">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="G25" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>276</v>
-      </c>
-      <c r="B26" t="s">
-        <v>277</v>
-      </c>
-      <c r="C26" t="s">
-        <v>278</v>
-      </c>
-      <c r="D26" t="s">
-        <v>2</v>
-      </c>
-      <c r="E26" t="s">
-        <v>184</v>
-      </c>
-      <c r="F26">
-        <v>0.8</v>
-      </c>
-      <c r="G26" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
lessons: publish Vav (letter 6)
Weekly limit cleared (2 lessons this ISO week: He + Vav, of 3 max);
owner approved. Editorial review applied all corrections via existing
rules (vowel-length x3, always/never, intra-lesson contradiction) with
no new owner decisions. Shortened the meta description from 169 to
152 chars during the double-check pass (over the 155-char cap).
Flips editorial/publication flags, registers Vav as published in the
SEO core, links it from the alphabet guide, and updates the hub
test's published-lesson assertions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8111" uniqueCount="943">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8120" uniqueCount="947">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
@@ -2726,6 +2726,18 @@
   </si>
   <si>
     <t>he hebrew letter; hebrew he pronunciation; hebrew letter he sound; learn hebrew letter he; he hebrew letter exercises; he vs chet hebrew letters; he at end of hebrew word</t>
+  </si>
+  <si>
+    <t>Vav Hebrew Letter (ו): Sound &amp; Vowels</t>
+  </si>
+  <si>
+    <t>Vav Hebrew Letter (ו): Sound, Vowels &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Vav (ו): its [v] sound, the Holam Male and Shuruk vowels ([o]/[u]), and words like דוֹב (bear) and דוּד (boiler), plus practice.</t>
+  </si>
+  <si>
+    <t>hebrew vav pronunciation; hebrew letter vav sound; learn hebrew letter vav; vav hebrew letter exercises; waw hebrew letter; vav with holam; vav with shuruk</t>
   </si>
   <si>
     <t>Hebrew Phrases for Beginners: 30 Useful Phrases | HebrewEdu</t>
@@ -3786,7 +3798,7 @@
         <v>96</v>
       </c>
       <c r="G16" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H16" t="s">
         <v>30</v>
@@ -15980,7 +15992,7 @@
         <v>306</v>
       </c>
       <c r="L177" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M177" t="s">
         <v>30</v>
@@ -16039,7 +16051,7 @@
         <v>306</v>
       </c>
       <c r="L178" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M178" t="s">
         <v>312</v>
@@ -16098,7 +16110,7 @@
         <v>306</v>
       </c>
       <c r="L179" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M179" t="s">
         <v>312</v>
@@ -16157,7 +16169,7 @@
         <v>306</v>
       </c>
       <c r="L180" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M180" t="s">
         <v>312</v>
@@ -16216,7 +16228,7 @@
         <v>306</v>
       </c>
       <c r="L181" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M181" t="s">
         <v>312</v>
@@ -16275,7 +16287,7 @@
         <v>306</v>
       </c>
       <c r="L182" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M182" t="s">
         <v>312</v>
@@ -16334,7 +16346,7 @@
         <v>306</v>
       </c>
       <c r="L183" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M183" t="s">
         <v>312</v>
@@ -16393,7 +16405,7 @@
         <v>306</v>
       </c>
       <c r="L184" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M184" t="s">
         <v>312</v>
@@ -26456,7 +26468,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -27743,7 +27755,7 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>282</v>
+        <v>96</v>
       </c>
       <c r="B28" t="s">
         <v>903</v>
@@ -27755,10 +27767,10 @@
         <v>905</v>
       </c>
       <c r="E28" t="s">
-        <v>279</v>
+        <v>92</v>
       </c>
       <c r="F28" t="s">
-        <v>755</v>
+        <v>93</v>
       </c>
       <c r="G28" t="s">
         <v>906</v>
@@ -27790,7 +27802,7 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>203</v>
+        <v>282</v>
       </c>
       <c r="B29" t="s">
         <v>907</v>
@@ -27802,10 +27814,10 @@
         <v>909</v>
       </c>
       <c r="E29" t="s">
-        <v>201</v>
+        <v>279</v>
       </c>
       <c r="F29" t="s">
-        <v>202</v>
+        <v>755</v>
       </c>
       <c r="G29" t="s">
         <v>910</v>
@@ -27829,7 +27841,7 @@
         <v>2</v>
       </c>
       <c r="N29" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O29" t="s">
         <v>29</v>
@@ -27837,7 +27849,7 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>171</v>
+        <v>203</v>
       </c>
       <c r="B30" t="s">
         <v>911</v>
@@ -27849,10 +27861,10 @@
         <v>913</v>
       </c>
       <c r="E30" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="F30" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="G30" t="s">
         <v>914</v>
@@ -27884,7 +27896,7 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>228</v>
+        <v>171</v>
       </c>
       <c r="B31" t="s">
         <v>915</v>
@@ -27896,10 +27908,10 @@
         <v>917</v>
       </c>
       <c r="E31" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="F31" t="s">
-        <v>257</v>
+        <v>169</v>
       </c>
       <c r="G31" t="s">
         <v>918</v>
@@ -27931,7 +27943,7 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>286</v>
+        <v>228</v>
       </c>
       <c r="B32" t="s">
         <v>919</v>
@@ -27943,10 +27955,10 @@
         <v>921</v>
       </c>
       <c r="E32" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F32" t="s">
-        <v>763</v>
+        <v>257</v>
       </c>
       <c r="G32" t="s">
         <v>922</v>
@@ -27970,7 +27982,7 @@
         <v>2</v>
       </c>
       <c r="N32" t="s">
-        <v>882</v>
+        <v>791</v>
       </c>
       <c r="O32" t="s">
         <v>29</v>
@@ -27978,46 +27990,46 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>286</v>
+      </c>
+      <c r="B33" t="s">
         <v>923</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>924</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>925</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
+        <v>283</v>
+      </c>
+      <c r="F33" t="s">
+        <v>763</v>
+      </c>
+      <c r="G33" t="s">
         <v>926</v>
       </c>
-      <c r="E33" t="s">
-        <v>2</v>
-      </c>
-      <c r="F33" t="s">
-        <v>2</v>
-      </c>
-      <c r="G33" t="s">
-        <v>2</v>
-      </c>
       <c r="H33" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I33" t="s">
-        <v>492</v>
+        <v>2</v>
       </c>
       <c r="J33" t="s">
-        <v>927</v>
+        <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="L33" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="M33" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N33" t="s">
-        <v>791</v>
+        <v>882</v>
       </c>
       <c r="O33" t="s">
         <v>29</v>
@@ -28025,16 +28037,16 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>927</v>
+      </c>
+      <c r="B34" t="s">
         <v>928</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>929</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>930</v>
-      </c>
-      <c r="D34" t="s">
-        <v>931</v>
       </c>
       <c r="E34" t="s">
         <v>2</v>
@@ -28049,19 +28061,19 @@
         <v>80</v>
       </c>
       <c r="I34" t="s">
-        <v>415</v>
+        <v>492</v>
       </c>
       <c r="J34" t="s">
-        <v>353</v>
+        <v>931</v>
       </c>
       <c r="K34" t="s">
         <v>80</v>
       </c>
       <c r="L34" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M34" t="s">
-        <v>932</v>
+        <v>64</v>
       </c>
       <c r="N34" t="s">
         <v>791</v>
@@ -28072,48 +28084,95 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>932</v>
+      </c>
+      <c r="B35" t="s">
         <v>933</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>934</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>935</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
+        <v>2</v>
+      </c>
+      <c r="F35" t="s">
+        <v>2</v>
+      </c>
+      <c r="G35" t="s">
+        <v>2</v>
+      </c>
+      <c r="H35" t="s">
+        <v>80</v>
+      </c>
+      <c r="I35" t="s">
+        <v>415</v>
+      </c>
+      <c r="J35" t="s">
+        <v>353</v>
+      </c>
+      <c r="K35" t="s">
+        <v>80</v>
+      </c>
+      <c r="L35" t="s">
+        <v>95</v>
+      </c>
+      <c r="M35" t="s">
         <v>936</v>
-      </c>
-      <c r="E35" t="s">
-        <v>2</v>
-      </c>
-      <c r="F35" t="s">
-        <v>2</v>
-      </c>
-      <c r="G35" t="s">
-        <v>2</v>
-      </c>
-      <c r="H35" t="s">
-        <v>2</v>
-      </c>
-      <c r="I35" t="s">
-        <v>2</v>
-      </c>
-      <c r="J35" t="s">
-        <v>2</v>
-      </c>
-      <c r="K35" t="s">
-        <v>2</v>
-      </c>
-      <c r="L35" t="s">
-        <v>2</v>
-      </c>
-      <c r="M35" t="s">
-        <v>2</v>
       </c>
       <c r="N35" t="s">
         <v>791</v>
       </c>
       <c r="O35" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>937</v>
+      </c>
+      <c r="B36" t="s">
+        <v>938</v>
+      </c>
+      <c r="C36" t="s">
+        <v>939</v>
+      </c>
+      <c r="D36" t="s">
+        <v>940</v>
+      </c>
+      <c r="E36" t="s">
+        <v>2</v>
+      </c>
+      <c r="F36" t="s">
+        <v>2</v>
+      </c>
+      <c r="G36" t="s">
+        <v>2</v>
+      </c>
+      <c r="H36" t="s">
+        <v>2</v>
+      </c>
+      <c r="I36" t="s">
+        <v>2</v>
+      </c>
+      <c r="J36" t="s">
+        <v>2</v>
+      </c>
+      <c r="K36" t="s">
+        <v>2</v>
+      </c>
+      <c r="L36" t="s">
+        <v>2</v>
+      </c>
+      <c r="M36" t="s">
+        <v>2</v>
+      </c>
+      <c r="N36" t="s">
+        <v>791</v>
+      </c>
+      <c r="O36" t="s">
         <v>29</v>
       </c>
     </row>
@@ -28126,7 +28185,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -28153,7 +28212,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -28276,22 +28335,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s">
         <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E7" t="s">
         <v>37</v>
       </c>
       <c r="F7">
-        <v>21.8</v>
+        <v>19.8</v>
       </c>
       <c r="G7" t="s">
         <v>30</v>
@@ -28299,22 +28358,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="B8" t="s">
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>62</v>
       </c>
       <c r="D8" t="s">
-        <v>103</v>
+        <v>65</v>
       </c>
       <c r="E8" t="s">
         <v>37</v>
       </c>
       <c r="F8">
-        <v>19.8</v>
+        <v>18.6</v>
       </c>
       <c r="G8" t="s">
         <v>30</v>
@@ -28322,22 +28381,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
         <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="D9" t="s">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="E9" t="s">
         <v>37</v>
       </c>
       <c r="F9">
-        <v>18.6</v>
+        <v>17.8</v>
       </c>
       <c r="G9" t="s">
         <v>30</v>
@@ -28345,22 +28404,22 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="B10" t="s">
         <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="E10" t="s">
         <v>37</v>
       </c>
       <c r="F10">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="G10" t="s">
         <v>30</v>
@@ -28368,22 +28427,22 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="B11" t="s">
         <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="D11" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="E11" t="s">
         <v>37</v>
       </c>
       <c r="F11">
-        <v>17.4</v>
+        <v>16</v>
       </c>
       <c r="G11" t="s">
         <v>30</v>
@@ -28391,22 +28450,22 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>134</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>135</v>
       </c>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>138</v>
       </c>
       <c r="E12" t="s">
         <v>37</v>
       </c>
       <c r="F12">
-        <v>16</v>
+        <v>13.9</v>
       </c>
       <c r="G12" t="s">
         <v>30</v>
@@ -28414,16 +28473,16 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D13" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E13" t="s">
         <v>37</v>
@@ -28437,16 +28496,16 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D14" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E14" t="s">
         <v>37</v>
@@ -28460,22 +28519,22 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D15" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
       </c>
       <c r="F15">
-        <v>13.9</v>
+        <v>13.3</v>
       </c>
       <c r="G15" t="s">
         <v>30</v>
@@ -28483,22 +28542,22 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="B16" t="s">
         <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="D16" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
       </c>
       <c r="F16">
-        <v>13.3</v>
+        <v>12.3</v>
       </c>
       <c r="G16" t="s">
         <v>30</v>
@@ -28506,22 +28565,22 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="D17" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="E17" t="s">
         <v>37</v>
       </c>
       <c r="F17">
-        <v>12.3</v>
+        <v>10.3</v>
       </c>
       <c r="G17" t="s">
         <v>30</v>
@@ -28529,22 +28588,22 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>154</v>
+        <v>273</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>274</v>
       </c>
       <c r="C18" t="s">
-        <v>155</v>
+        <v>275</v>
       </c>
       <c r="D18" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="E18" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F18">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="G18" t="s">
         <v>30</v>
@@ -28552,16 +28611,16 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="B19" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="C19" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="D19" t="s">
-        <v>143</v>
+        <v>286</v>
       </c>
       <c r="E19" t="s">
         <v>184</v>
@@ -28575,22 +28634,22 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="B20" t="s">
-        <v>284</v>
+        <v>32</v>
       </c>
       <c r="C20" t="s">
-        <v>285</v>
+        <v>159</v>
       </c>
       <c r="D20" t="s">
-        <v>286</v>
+        <v>161</v>
       </c>
       <c r="E20" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F20">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G20" t="s">
         <v>30</v>
@@ -28598,22 +28657,22 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>181</v>
       </c>
       <c r="C21" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="D21" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="E21" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F21">
-        <v>9</v>
+        <v>8.3</v>
       </c>
       <c r="G21" t="s">
         <v>30</v>
@@ -28621,22 +28680,22 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>180</v>
+        <v>267</v>
       </c>
       <c r="B22" t="s">
-        <v>181</v>
+        <v>268</v>
       </c>
       <c r="C22" t="s">
-        <v>182</v>
+        <v>269</v>
       </c>
       <c r="D22" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="E22" t="s">
         <v>184</v>
       </c>
       <c r="F22">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G22" t="s">
         <v>30</v>
@@ -28644,16 +28703,16 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B23" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C23" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D23" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="E23" t="s">
         <v>184</v>
@@ -28667,47 +28726,24 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B24" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="C24" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D24" t="s">
-        <v>247</v>
+        <v>2</v>
       </c>
       <c r="E24" t="s">
         <v>184</v>
       </c>
       <c r="F24">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="G24" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>276</v>
-      </c>
-      <c r="B25" t="s">
-        <v>277</v>
-      </c>
-      <c r="C25" t="s">
-        <v>278</v>
-      </c>
-      <c r="D25" t="s">
-        <v>2</v>
-      </c>
-      <c r="E25" t="s">
-        <v>184</v>
-      </c>
-      <c r="F25">
-        <v>0.8</v>
-      </c>
-      <c r="G25" t="s">
         <v>30</v>
       </c>
     </row>
@@ -28758,27 +28794,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>938</v>
+        <v>942</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>939</v>
+        <v>943</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>940</v>
+        <v>944</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Chet letter lesson (EN + FR)
Normalizes the eighth letter lesson from its pinned raw snapshots in
both locales. Editorial review: the furtive-Patah STRIPED_BLOCK is held
out (no renderer yet; the concept stays in three exercise tips), EN
"Final Chet" becomes "Chet at the end of the word" (new rule in the
editorial rules), EN meta trimmed to 151 characters, FR "ch" -> "kh"
transliteration via the new override paths. Registers SEO (EN and FR
clusters/keywords planned -> published, pages rows), links it from the
alphabet guide, and publishes both locales on 2026-10-23.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,12 +17,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10595" uniqueCount="1235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10615" uniqueCount="1241">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
   <si>
-    <t>Generated: 2026-10-21 by scripts/seo/build-core.mjs (npm run seo:build)</t>
+    <t>Generated: 2026-10-23 by scripts/seo/build-core.mjs (npm run seo:build)</t>
   </si>
   <si>
     <t/>
@@ -3409,6 +3409,18 @@
     <t>hebrew zayin pronunciation; hebrew letter zayin sound; learn hebrew letter zayin; zayin hebrew letter exercises; zain hebrew letter; how to recognize zayin</t>
   </si>
   <si>
+    <t>Chet Hebrew Letter (ח): Sound &amp; Furtive Patah</t>
+  </si>
+  <si>
+    <t>Chet Hebrew Letter (ח): Sound, Furtive Patah &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Chet (ח): its guttural [ch] sound, the furtive Patah in כּוֹחַ (strength), words like אָח (brother), plus interactive practice.</t>
+  </si>
+  <si>
+    <t>hebrew chet pronunciation; hebrew letter chet sound; learn hebrew letter chet; chet hebrew letter exercises; het hebrew letter; chet vs he hebrew letters</t>
+  </si>
+  <si>
     <t>Hebrew Phrases for Beginners: 30 Useful Phrases</t>
   </si>
   <si>
@@ -3584,6 +3596,12 @@
   </si>
   <si>
     <t>Apprends la lettre hébraïque Zayin (ז) et son son [z], avec des mots comme זְבוּב (mouche) et זֶה (ceci), ainsi que des exercices interactifs.</t>
+  </si>
+  <si>
+    <t>Heth (ח) : lettre hébraïque, son et exemples</t>
+  </si>
+  <si>
+    <t>Apprends la lettre hébraïque Heth (ח) et son son guttural [kh], avec des mots comme אָח (frère) et חַג (fête), ainsi que des exercices interactifs.</t>
   </si>
   <si>
     <t>Phrases et expressions en hébreu pour débutants</t>
@@ -4981,7 +4999,7 @@
         <v>138</v>
       </c>
       <c r="G27" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H27" t="s">
         <v>30</v>
@@ -6924,7 +6942,7 @@
         <v>350</v>
       </c>
       <c r="G94" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H94" t="s">
         <v>306</v>
@@ -19445,7 +19463,7 @@
         <v>453</v>
       </c>
       <c r="L192" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M192" t="s">
         <v>30</v>
@@ -19507,7 +19525,7 @@
         <v>453</v>
       </c>
       <c r="L193" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M193" t="s">
         <v>306</v>
@@ -19569,7 +19587,7 @@
         <v>453</v>
       </c>
       <c r="L194" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M194" t="s">
         <v>306</v>
@@ -19631,7 +19649,7 @@
         <v>453</v>
       </c>
       <c r="L195" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M195" t="s">
         <v>306</v>
@@ -19693,7 +19711,7 @@
         <v>453</v>
       </c>
       <c r="L196" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M196" t="s">
         <v>306</v>
@@ -19755,7 +19773,7 @@
         <v>453</v>
       </c>
       <c r="L197" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M197" t="s">
         <v>306</v>
@@ -19817,7 +19835,7 @@
         <v>453</v>
       </c>
       <c r="L198" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M198" t="s">
         <v>306</v>
@@ -30853,7 +30871,7 @@
         <v>460</v>
       </c>
       <c r="L376" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M376" t="s">
         <v>306</v>
@@ -33369,7 +33387,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P62"/>
+  <dimension ref="A1:P64"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -34837,7 +34855,7 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>282</v>
+        <v>138</v>
       </c>
       <c r="B30" t="s">
         <v>1130</v>
@@ -34849,10 +34867,10 @@
         <v>1132</v>
       </c>
       <c r="E30" t="s">
-        <v>279</v>
+        <v>134</v>
       </c>
       <c r="F30" t="s">
-        <v>899</v>
+        <v>135</v>
       </c>
       <c r="G30" t="s">
         <v>1133</v>
@@ -34887,7 +34905,7 @@
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>203</v>
+        <v>282</v>
       </c>
       <c r="B31" t="s">
         <v>1134</v>
@@ -34899,10 +34917,10 @@
         <v>1136</v>
       </c>
       <c r="E31" t="s">
-        <v>201</v>
+        <v>279</v>
       </c>
       <c r="F31" t="s">
-        <v>202</v>
+        <v>899</v>
       </c>
       <c r="G31" t="s">
         <v>1137</v>
@@ -34926,7 +34944,7 @@
         <v>2</v>
       </c>
       <c r="N31" t="s">
-        <v>1021</v>
+        <v>1101</v>
       </c>
       <c r="O31" t="s">
         <v>29</v>
@@ -34937,7 +34955,7 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>171</v>
+        <v>203</v>
       </c>
       <c r="B32" t="s">
         <v>1138</v>
@@ -34949,10 +34967,10 @@
         <v>1140</v>
       </c>
       <c r="E32" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="F32" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="G32" t="s">
         <v>1141</v>
@@ -34987,7 +35005,7 @@
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>228</v>
+        <v>171</v>
       </c>
       <c r="B33" t="s">
         <v>1142</v>
@@ -34999,10 +35017,10 @@
         <v>1144</v>
       </c>
       <c r="E33" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="F33" t="s">
-        <v>257</v>
+        <v>169</v>
       </c>
       <c r="G33" t="s">
         <v>1145</v>
@@ -35037,7 +35055,7 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>286</v>
+        <v>228</v>
       </c>
       <c r="B34" t="s">
         <v>1146</v>
@@ -35049,10 +35067,10 @@
         <v>1148</v>
       </c>
       <c r="E34" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F34" t="s">
-        <v>907</v>
+        <v>257</v>
       </c>
       <c r="G34" t="s">
         <v>1149</v>
@@ -35076,7 +35094,7 @@
         <v>2</v>
       </c>
       <c r="N34" t="s">
-        <v>1101</v>
+        <v>1021</v>
       </c>
       <c r="O34" t="s">
         <v>29</v>
@@ -35087,10 +35105,10 @@
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>286</v>
+      </c>
+      <c r="B35" t="s">
         <v>1150</v>
-      </c>
-      <c r="B35" t="s">
-        <v>1151</v>
       </c>
       <c r="C35" t="s">
         <v>1151</v>
@@ -35099,34 +35117,34 @@
         <v>1152</v>
       </c>
       <c r="E35" t="s">
-        <v>2</v>
+        <v>283</v>
       </c>
       <c r="F35" t="s">
-        <v>2</v>
+        <v>907</v>
       </c>
       <c r="G35" t="s">
-        <v>2</v>
+        <v>1153</v>
       </c>
       <c r="H35" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I35" t="s">
-        <v>636</v>
+        <v>2</v>
       </c>
       <c r="J35" t="s">
-        <v>1153</v>
+        <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="L35" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="M35" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N35" t="s">
-        <v>1021</v>
+        <v>1101</v>
       </c>
       <c r="O35" t="s">
         <v>29</v>
@@ -35161,19 +35179,19 @@
         <v>80</v>
       </c>
       <c r="I36" t="s">
-        <v>561</v>
+        <v>636</v>
       </c>
       <c r="J36" t="s">
-        <v>499</v>
+        <v>1157</v>
       </c>
       <c r="K36" t="s">
         <v>80</v>
       </c>
       <c r="L36" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M36" t="s">
-        <v>1157</v>
+        <v>64</v>
       </c>
       <c r="N36" t="s">
         <v>1021</v>
@@ -35208,22 +35226,22 @@
         <v>2</v>
       </c>
       <c r="H37" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="I37" t="s">
-        <v>2</v>
+        <v>561</v>
       </c>
       <c r="J37" t="s">
-        <v>2</v>
+        <v>499</v>
       </c>
       <c r="K37" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="L37" t="s">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="M37" t="s">
-        <v>2</v>
+        <v>1161</v>
       </c>
       <c r="N37" t="s">
         <v>1021</v>
@@ -35237,22 +35255,22 @@
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>301</v>
+        <v>1162</v>
       </c>
       <c r="B38" t="s">
-        <v>1161</v>
+        <v>1163</v>
       </c>
       <c r="C38" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="D38" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="E38" t="s">
-        <v>298</v>
+        <v>2</v>
       </c>
       <c r="F38" t="s">
-        <v>300</v>
+        <v>2</v>
       </c>
       <c r="G38" t="s">
         <v>2</v>
@@ -35276,36 +35294,36 @@
         <v>2</v>
       </c>
       <c r="N38" t="s">
-        <v>2</v>
+        <v>1021</v>
       </c>
       <c r="O38" t="s">
         <v>29</v>
       </c>
       <c r="P38" t="s">
-        <v>922</v>
+        <v>457</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="B39" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="C39" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="D39" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="E39" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="F39" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="G39" t="s">
-        <v>929</v>
+        <v>2</v>
       </c>
       <c r="H39" t="s">
         <v>2</v>
@@ -35337,25 +35355,25 @@
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>320</v>
+        <v>292</v>
       </c>
       <c r="B40" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="C40" t="s">
-        <v>1167</v>
+        <v>1169</v>
       </c>
       <c r="D40" t="s">
-        <v>1168</v>
+        <v>1170</v>
       </c>
       <c r="E40" t="s">
-        <v>317</v>
+        <v>287</v>
       </c>
       <c r="F40" t="s">
-        <v>1169</v>
+        <v>289</v>
       </c>
       <c r="G40" t="s">
-        <v>1170</v>
+        <v>929</v>
       </c>
       <c r="H40" t="s">
         <v>2</v>
@@ -35387,7 +35405,7 @@
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B41" t="s">
         <v>1171</v>
@@ -35399,7 +35417,7 @@
         <v>1172</v>
       </c>
       <c r="E41" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="F41" t="s">
         <v>1173</v>
@@ -35437,7 +35455,7 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>347</v>
+        <v>323</v>
       </c>
       <c r="B42" t="s">
         <v>1175</v>
@@ -35449,13 +35467,13 @@
         <v>1176</v>
       </c>
       <c r="E42" t="s">
-        <v>345</v>
+        <v>321</v>
       </c>
       <c r="F42" t="s">
         <v>1177</v>
       </c>
       <c r="G42" t="s">
-        <v>2</v>
+        <v>1178</v>
       </c>
       <c r="H42" t="s">
         <v>2</v>
@@ -35487,25 +35505,25 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="B43" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="C43" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="D43" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="E43" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="F43" t="s">
-        <v>337</v>
+        <v>1181</v>
       </c>
       <c r="G43" t="s">
-        <v>937</v>
+        <v>2</v>
       </c>
       <c r="H43" t="s">
         <v>2</v>
@@ -35537,25 +35555,25 @@
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="B44" t="s">
-        <v>1180</v>
+        <v>1182</v>
       </c>
       <c r="C44" t="s">
-        <v>1180</v>
+        <v>1182</v>
       </c>
       <c r="D44" t="s">
-        <v>1181</v>
+        <v>1183</v>
       </c>
       <c r="E44" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="F44" t="s">
-        <v>1182</v>
+        <v>337</v>
       </c>
       <c r="G44" t="s">
-        <v>328</v>
+        <v>937</v>
       </c>
       <c r="H44" t="s">
         <v>2</v>
@@ -35587,25 +35605,25 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B45" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="C45" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="D45" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="E45" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="F45" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="G45" t="s">
-        <v>1186</v>
+        <v>328</v>
       </c>
       <c r="H45" t="s">
         <v>2</v>
@@ -35637,7 +35655,7 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="B46" t="s">
         <v>1187</v>
@@ -35649,13 +35667,13 @@
         <v>1188</v>
       </c>
       <c r="E46" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="F46" t="s">
-        <v>331</v>
+        <v>1189</v>
       </c>
       <c r="G46" t="s">
-        <v>2</v>
+        <v>1190</v>
       </c>
       <c r="H46" t="s">
         <v>2</v>
@@ -35687,25 +35705,25 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>373</v>
+        <v>332</v>
       </c>
       <c r="B47" t="s">
-        <v>1189</v>
+        <v>1191</v>
       </c>
       <c r="C47" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="D47" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="E47" t="s">
-        <v>369</v>
+        <v>330</v>
       </c>
       <c r="F47" t="s">
-        <v>371</v>
+        <v>331</v>
       </c>
       <c r="G47" t="s">
-        <v>1192</v>
+        <v>2</v>
       </c>
       <c r="H47" t="s">
         <v>2</v>
@@ -35737,7 +35755,7 @@
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>297</v>
+        <v>350</v>
       </c>
       <c r="B48" t="s">
         <v>1193</v>
@@ -35749,13 +35767,13 @@
         <v>1194</v>
       </c>
       <c r="E48" t="s">
-        <v>293</v>
+        <v>348</v>
       </c>
       <c r="F48" t="s">
-        <v>295</v>
+        <v>349</v>
       </c>
       <c r="G48" t="s">
-        <v>1195</v>
+        <v>2</v>
       </c>
       <c r="H48" t="s">
         <v>2</v>
@@ -35787,10 +35805,10 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="B49" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C49" t="s">
         <v>1196</v>
@@ -35799,13 +35817,13 @@
         <v>1197</v>
       </c>
       <c r="E49" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="F49" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="G49" t="s">
-        <v>951</v>
+        <v>1198</v>
       </c>
       <c r="H49" t="s">
         <v>2</v>
@@ -35837,25 +35855,25 @@
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>383</v>
+        <v>297</v>
       </c>
       <c r="B50" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="C50" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="D50" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="E50" t="s">
-        <v>379</v>
+        <v>293</v>
       </c>
       <c r="F50" t="s">
-        <v>381</v>
+        <v>295</v>
       </c>
       <c r="G50" t="s">
-        <v>2</v>
+        <v>1201</v>
       </c>
       <c r="H50" t="s">
         <v>2</v>
@@ -35887,25 +35905,25 @@
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="B51" t="s">
-        <v>1200</v>
+        <v>1202</v>
       </c>
       <c r="C51" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="D51" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="E51" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="F51" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="G51" t="s">
-        <v>2</v>
+        <v>951</v>
       </c>
       <c r="H51" t="s">
         <v>2</v>
@@ -35937,25 +35955,25 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="B52" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="C52" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="D52" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="E52" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
       <c r="F52" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="G52" t="s">
-        <v>958</v>
+        <v>2</v>
       </c>
       <c r="H52" t="s">
         <v>2</v>
@@ -35987,25 +36005,25 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="B53" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="C53" t="s">
-        <v>1205</v>
+        <v>1207</v>
       </c>
       <c r="D53" t="s">
-        <v>1206</v>
+        <v>1208</v>
       </c>
       <c r="E53" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="F53" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="G53" t="s">
-        <v>1207</v>
+        <v>2</v>
       </c>
       <c r="H53" t="s">
         <v>2</v>
@@ -36037,25 +36055,25 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="B54" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="C54" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="D54" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="E54" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="F54" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="G54" t="s">
-        <v>1210</v>
+        <v>958</v>
       </c>
       <c r="H54" t="s">
         <v>2</v>
@@ -36087,7 +36105,7 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
       <c r="B55" t="s">
         <v>1211</v>
@@ -36099,10 +36117,10 @@
         <v>1212</v>
       </c>
       <c r="E55" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="F55" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="G55" t="s">
         <v>1213</v>
@@ -36137,7 +36155,7 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
       <c r="B56" t="s">
         <v>1214</v>
@@ -36149,13 +36167,13 @@
         <v>1215</v>
       </c>
       <c r="E56" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="F56" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="G56" t="s">
-        <v>979</v>
+        <v>1216</v>
       </c>
       <c r="H56" t="s">
         <v>2</v>
@@ -36187,25 +36205,25 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="B57" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="C57" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="D57" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="E57" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="F57" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="G57" t="s">
-        <v>982</v>
+        <v>1219</v>
       </c>
       <c r="H57" t="s">
         <v>2</v>
@@ -36237,25 +36255,25 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="B58" t="s">
-        <v>1218</v>
+        <v>1220</v>
       </c>
       <c r="C58" t="s">
-        <v>1218</v>
+        <v>1220</v>
       </c>
       <c r="D58" t="s">
-        <v>1219</v>
+        <v>1221</v>
       </c>
       <c r="E58" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="F58" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="G58" t="s">
-        <v>1220</v>
+        <v>979</v>
       </c>
       <c r="H58" t="s">
         <v>2</v>
@@ -36287,25 +36305,25 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="B59" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="C59" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="D59" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="E59" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="F59" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="G59" t="s">
-        <v>990</v>
+        <v>982</v>
       </c>
       <c r="H59" t="s">
         <v>2</v>
@@ -36337,25 +36355,25 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="B60" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="C60" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="D60" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="E60" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="F60" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="G60" t="s">
-        <v>994</v>
+        <v>1226</v>
       </c>
       <c r="H60" t="s">
         <v>2</v>
@@ -36387,25 +36405,25 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="B61" t="s">
-        <v>1225</v>
+        <v>1227</v>
       </c>
       <c r="C61" t="s">
-        <v>1225</v>
+        <v>1227</v>
       </c>
       <c r="D61" t="s">
-        <v>1226</v>
+        <v>1228</v>
       </c>
       <c r="E61" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="F61" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="G61" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="H61" t="s">
         <v>2</v>
@@ -36437,51 +36455,151 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>424</v>
+      </c>
+      <c r="B62" t="s">
+        <v>1229</v>
+      </c>
+      <c r="C62" t="s">
+        <v>1229</v>
+      </c>
+      <c r="D62" t="s">
+        <v>1230</v>
+      </c>
+      <c r="E62" t="s">
+        <v>421</v>
+      </c>
+      <c r="F62" t="s">
+        <v>423</v>
+      </c>
+      <c r="G62" t="s">
+        <v>994</v>
+      </c>
+      <c r="H62" t="s">
+        <v>2</v>
+      </c>
+      <c r="I62" t="s">
+        <v>2</v>
+      </c>
+      <c r="J62" t="s">
+        <v>2</v>
+      </c>
+      <c r="K62" t="s">
+        <v>2</v>
+      </c>
+      <c r="L62" t="s">
+        <v>2</v>
+      </c>
+      <c r="M62" t="s">
+        <v>2</v>
+      </c>
+      <c r="N62" t="s">
+        <v>2</v>
+      </c>
+      <c r="O62" t="s">
+        <v>29</v>
+      </c>
+      <c r="P62" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>428</v>
+      </c>
+      <c r="B63" t="s">
+        <v>1231</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1231</v>
+      </c>
+      <c r="D63" t="s">
+        <v>1232</v>
+      </c>
+      <c r="E63" t="s">
+        <v>425</v>
+      </c>
+      <c r="F63" t="s">
+        <v>427</v>
+      </c>
+      <c r="G63" t="s">
+        <v>994</v>
+      </c>
+      <c r="H63" t="s">
+        <v>2</v>
+      </c>
+      <c r="I63" t="s">
+        <v>2</v>
+      </c>
+      <c r="J63" t="s">
+        <v>2</v>
+      </c>
+      <c r="K63" t="s">
+        <v>2</v>
+      </c>
+      <c r="L63" t="s">
+        <v>2</v>
+      </c>
+      <c r="M63" t="s">
+        <v>2</v>
+      </c>
+      <c r="N63" t="s">
+        <v>2</v>
+      </c>
+      <c r="O63" t="s">
+        <v>29</v>
+      </c>
+      <c r="P63" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>432</v>
       </c>
-      <c r="B62" t="s">
-        <v>1227</v>
-      </c>
-      <c r="C62" t="s">
-        <v>1227</v>
-      </c>
-      <c r="D62" t="s">
-        <v>1228</v>
-      </c>
-      <c r="E62" t="s">
+      <c r="B64" t="s">
+        <v>1233</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1233</v>
+      </c>
+      <c r="D64" t="s">
+        <v>1234</v>
+      </c>
+      <c r="E64" t="s">
         <v>429</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F64" t="s">
         <v>431</v>
       </c>
-      <c r="G62" t="s">
+      <c r="G64" t="s">
         <v>1000</v>
       </c>
-      <c r="H62" t="s">
-        <v>2</v>
-      </c>
-      <c r="I62" t="s">
-        <v>2</v>
-      </c>
-      <c r="J62" t="s">
-        <v>2</v>
-      </c>
-      <c r="K62" t="s">
-        <v>2</v>
-      </c>
-      <c r="L62" t="s">
-        <v>2</v>
-      </c>
-      <c r="M62" t="s">
-        <v>2</v>
-      </c>
-      <c r="N62" t="s">
-        <v>2</v>
-      </c>
-      <c r="O62" t="s">
-        <v>29</v>
-      </c>
-      <c r="P62" t="s">
+      <c r="H64" t="s">
+        <v>2</v>
+      </c>
+      <c r="I64" t="s">
+        <v>2</v>
+      </c>
+      <c r="J64" t="s">
+        <v>2</v>
+      </c>
+      <c r="K64" t="s">
+        <v>2</v>
+      </c>
+      <c r="L64" t="s">
+        <v>2</v>
+      </c>
+      <c r="M64" t="s">
+        <v>2</v>
+      </c>
+      <c r="N64" t="s">
+        <v>2</v>
+      </c>
+      <c r="O64" t="s">
+        <v>29</v>
+      </c>
+      <c r="P64" t="s">
         <v>922</v>
       </c>
     </row>
@@ -36494,7 +36612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -36521,7 +36639,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1229</v>
+        <v>1235</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -36759,16 +36877,16 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D12" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E12" t="s">
         <v>37</v>
@@ -36782,16 +36900,16 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D13" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E13" t="s">
         <v>37</v>
@@ -36805,22 +36923,22 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>121</v>
       </c>
       <c r="D14" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="E14" t="s">
         <v>37</v>
       </c>
       <c r="F14">
-        <v>13.9</v>
+        <v>12.3</v>
       </c>
       <c r="G14" t="s">
         <v>30</v>
@@ -36828,22 +36946,22 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="D15" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
       </c>
       <c r="F15">
-        <v>12.3</v>
+        <v>10.3</v>
       </c>
       <c r="G15" t="s">
         <v>30</v>
@@ -36851,16 +36969,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>154</v>
+        <v>302</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>303</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>304</v>
       </c>
       <c r="D16" t="s">
-        <v>157</v>
+        <v>305</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
@@ -36869,44 +36987,44 @@
         <v>10.3</v>
       </c>
       <c r="G16" t="s">
-        <v>30</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>302</v>
+        <v>273</v>
       </c>
       <c r="B17" t="s">
-        <v>303</v>
+        <v>274</v>
       </c>
       <c r="C17" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="D17" t="s">
-        <v>305</v>
+        <v>143</v>
       </c>
       <c r="E17" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F17">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="G17" t="s">
-        <v>306</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="B18" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="C18" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="D18" t="s">
-        <v>143</v>
+        <v>286</v>
       </c>
       <c r="E18" t="s">
         <v>184</v>
@@ -36920,45 +37038,45 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>283</v>
+        <v>307</v>
       </c>
       <c r="B19" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="C19" t="s">
-        <v>285</v>
+        <v>308</v>
       </c>
       <c r="D19" t="s">
-        <v>286</v>
+        <v>309</v>
       </c>
       <c r="E19" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F19">
-        <v>10</v>
+        <v>9.8</v>
       </c>
       <c r="G19" t="s">
-        <v>30</v>
+        <v>306</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B20" t="s">
         <v>303</v>
       </c>
       <c r="C20" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D20" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="E20" t="s">
         <v>37</v>
       </c>
       <c r="F20">
-        <v>9.8</v>
+        <v>9.3</v>
       </c>
       <c r="G20" t="s">
         <v>306</v>
@@ -36966,16 +37084,16 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="B21" t="s">
         <v>303</v>
       </c>
       <c r="C21" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="D21" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="E21" t="s">
         <v>37</v>
@@ -36989,45 +37107,45 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>314</v>
+        <v>158</v>
       </c>
       <c r="B22" t="s">
-        <v>303</v>
+        <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>315</v>
+        <v>159</v>
       </c>
       <c r="D22" t="s">
-        <v>316</v>
+        <v>161</v>
       </c>
       <c r="E22" t="s">
         <v>37</v>
       </c>
       <c r="F22">
-        <v>9.3</v>
+        <v>9</v>
       </c>
       <c r="G22" t="s">
-        <v>306</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>181</v>
       </c>
       <c r="C23" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="D23" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="E23" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F23">
-        <v>9</v>
+        <v>8.3</v>
       </c>
       <c r="G23" t="s">
         <v>30</v>
@@ -37035,39 +37153,39 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>180</v>
+        <v>333</v>
       </c>
       <c r="B24" t="s">
-        <v>181</v>
+        <v>303</v>
       </c>
       <c r="C24" t="s">
-        <v>182</v>
+        <v>334</v>
       </c>
       <c r="D24" t="s">
-        <v>183</v>
+        <v>335</v>
       </c>
       <c r="E24" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F24">
         <v>8.3</v>
       </c>
       <c r="G24" t="s">
-        <v>30</v>
+        <v>306</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B25" t="s">
         <v>303</v>
       </c>
       <c r="C25" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D25" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E25" t="s">
         <v>37</v>
@@ -37081,16 +37199,16 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B26" t="s">
         <v>303</v>
       </c>
       <c r="C26" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D26" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E26" t="s">
         <v>37</v>
@@ -37104,39 +37222,39 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>342</v>
+        <v>267</v>
       </c>
       <c r="B27" t="s">
-        <v>303</v>
+        <v>268</v>
       </c>
       <c r="C27" t="s">
-        <v>343</v>
+        <v>269</v>
       </c>
       <c r="D27" t="s">
-        <v>344</v>
+        <v>194</v>
       </c>
       <c r="E27" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F27">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G27" t="s">
-        <v>306</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B28" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C28" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D28" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="E28" t="s">
         <v>184</v>
@@ -37150,39 +37268,39 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>270</v>
+        <v>351</v>
       </c>
       <c r="B29" t="s">
-        <v>271</v>
+        <v>303</v>
       </c>
       <c r="C29" t="s">
-        <v>272</v>
+        <v>352</v>
       </c>
       <c r="D29" t="s">
-        <v>247</v>
+        <v>353</v>
       </c>
       <c r="E29" t="s">
-        <v>184</v>
+        <v>37</v>
       </c>
       <c r="F29">
         <v>8</v>
       </c>
       <c r="G29" t="s">
-        <v>30</v>
+        <v>306</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="B30" t="s">
         <v>303</v>
       </c>
       <c r="C30" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="D30" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="E30" t="s">
         <v>37</v>
@@ -37196,16 +37314,16 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="B31" t="s">
         <v>303</v>
       </c>
       <c r="C31" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="D31" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="E31" t="s">
         <v>37</v>
@@ -37219,16 +37337,16 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="B32" t="s">
         <v>303</v>
       </c>
       <c r="C32" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="D32" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="E32" t="s">
         <v>37</v>
@@ -37242,16 +37360,16 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="B33" t="s">
         <v>303</v>
       </c>
       <c r="C33" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="D33" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="E33" t="s">
         <v>37</v>
@@ -37265,16 +37383,16 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="B34" t="s">
         <v>303</v>
       </c>
       <c r="C34" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="D34" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="E34" t="s">
         <v>37</v>
@@ -37288,70 +37406,24 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>363</v>
+        <v>276</v>
       </c>
       <c r="B35" t="s">
-        <v>303</v>
+        <v>277</v>
       </c>
       <c r="C35" t="s">
-        <v>364</v>
+        <v>278</v>
       </c>
       <c r="D35" t="s">
-        <v>365</v>
+        <v>2</v>
       </c>
       <c r="E35" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="F35">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="G35" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>366</v>
-      </c>
-      <c r="B36" t="s">
-        <v>303</v>
-      </c>
-      <c r="C36" t="s">
-        <v>367</v>
-      </c>
-      <c r="D36" t="s">
-        <v>368</v>
-      </c>
-      <c r="E36" t="s">
-        <v>37</v>
-      </c>
-      <c r="F36">
-        <v>8</v>
-      </c>
-      <c r="G36" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>276</v>
-      </c>
-      <c r="B37" t="s">
-        <v>277</v>
-      </c>
-      <c r="C37" t="s">
-        <v>278</v>
-      </c>
-      <c r="D37" t="s">
-        <v>2</v>
-      </c>
-      <c r="E37" t="s">
-        <v>184</v>
-      </c>
-      <c r="F37">
-        <v>0.8</v>
-      </c>
-      <c r="G37" t="s">
         <v>30</v>
       </c>
     </row>
@@ -37402,27 +37474,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>1230</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1231</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1232</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1233</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1234</v>
+        <v>1240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Drop the last title brand suffixes; guide description answers "hebrew alphabet"
- /blog/hebrew-alphabet-complete-guide/, /play/ and /play/alef-bet-rush/
  lose "| HebrewEdu" / "| HebrewEdu Blog" (owner-approved), which empties
  check-i18n's BRAND_SUFFIX_ALLOWLIST and TITLE_LENGTH_ALLOWLIST.
- Guide seoTitle now leads with "Hebrew Alphabet"; its meta description
  states the 22 letters, shapes, names, sounds, final forms and nikud.
- docs/I18N.md known gaps and docs/seo/core/pages.csv updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -3205,13 +3205,13 @@
     <t>hebrew comprehensible input; hebrew listening practice for beginners</t>
   </si>
   <si>
-    <t>The Hebrew Alphabet: A Complete Guide to All 22 Letters | HebrewEdu Blog</t>
+    <t>Hebrew Alphabet: A Complete Guide to All 22 Letters</t>
   </si>
   <si>
     <t>The Hebrew Alphabet: A Complete Guide to All 22 Letters</t>
   </si>
   <si>
-    <t>Everything you need to know about the Hebrew alphabet — letter shapes, names, sounds, and practical tips for learning Aleph Bet from scratch.</t>
+    <t>The Hebrew alphabet has 22 letters. See each letter's shape, name and sound, the five final forms, nikud vowels and tips to learn the Aleph Bet.</t>
   </si>
   <si>
     <t>hebrew alphabet; how many letters are in the hebrew alphabet; hebrew alphabet pronunciation; how to read hebrew; learn hebrew alphabet; learning the hebrew alphabet; learn aleph bet; alephbet; hebrew alphabet letter names; hebrew final letters; hebrew reading direction; learn hebrew alphabet online; how to pronounce chet in hebrew; how to pronounce resh in hebrew; hebrew capital and lowercase letters; bet vs vet pronunciation; shin vs sin pronunciation; kaf vs chaf pronunciation; vav vowel and consonant sounds; yod vowel and consonant sounds; learn hebrew aleph bet; learning hebrew alphabet; learn hebrew letters; learn hebrew alef bet; how to learn hebrew alphabet; hebrew aleph bet; learn hebrew script; learning hebrew letters; aleph bet; hebrew alef bet; how to learn hebrew letters; aleph bet hebrew; easy way to learn hebrew alphabet; hebrew alphabet learn</t>
@@ -3523,7 +3523,7 @@
     <t>useful hebrew phrases; common hebrew phrases</t>
   </si>
   <si>
-    <t>Free Hebrew Learning Games Online | HebrewEdu</t>
+    <t>Free Hebrew Learning Games Online</t>
   </si>
   <si>
     <t>Free Hebrew Learning Games for Beginners</t>
@@ -3535,7 +3535,7 @@
     <t>free hebrew learning games; hebrew alphabet game no download; hebrew alphabet game no sign up; learn hebrew alphabet game; aleph bet games online</t>
   </si>
   <si>
-    <t>Hebrew Alphabet Game: Learn the Alef Bet | HebrewEdu</t>
+    <t>Hebrew Alphabet Game: Learn the Alef Bet</t>
   </si>
   <si>
     <t>Alef Bet Rush: Free Hebrew Alphabet Game</t>

</xml_diff>

<commit_message>
Add Tet letter lesson (EN + FR)
Normalizes the ninth letter lesson from its pinned raw snapshots in both
locales, no holdouts. Editorial review: "final Bet/Chet" becomes "at the
end of the word" in both locales, the "Correct!"/"Exact !" opener is
dropped from the Q11 tip (new rule: tips show after wrong answers too),
FR "ch" -> "kh" for בֶּטַח, and the intro now says Tet sounds like Tav
in Modern Hebrew (owner decision). Registers SEO (EN and FR clusters and
keywords planned -> published, pages rows), links it from the alphabet
guide, and publishes both locales on 2026-10-26.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,12 +17,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12142" uniqueCount="1412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12162" uniqueCount="1418">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
   <si>
-    <t>Generated: 2026-10-25 by scripts/seo/build-core.mjs (npm run seo:build)</t>
+    <t>Generated: 2026-10-26 by scripts/seo/build-core.mjs (npm run seo:build)</t>
   </si>
   <si>
     <t/>
@@ -3877,6 +3877,18 @@
     <t>hebrew chet pronunciation; hebrew letter chet sound; learn hebrew letter chet; chet hebrew letter exercises; het hebrew letter; chet vs he hebrew letters</t>
   </si>
   <si>
+    <t>Tet Hebrew Letter (ט): Sound &amp; Words</t>
+  </si>
+  <si>
+    <t>Tet Hebrew Letter (ט): Sound, Words &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Tet (ט): its [t] sound, its traditional link to טוֹב (good), words like בֶּטַח (sure), plus interactive practice.</t>
+  </si>
+  <si>
+    <t>hebrew tet pronunciation; hebrew letter tet sound; learn hebrew letter tet; tet hebrew letter exercises; teth hebrew letter; tet vs tav hebrew pronunciation</t>
+  </si>
+  <si>
     <t>Hebrew Phrases for Beginners: 30 Useful Phrases</t>
   </si>
   <si>
@@ -4058,6 +4070,12 @@
   </si>
   <si>
     <t>Apprends la lettre hébraïque Heth (ח) et son son guttural [kh], avec des mots comme אָח (frère) et חַג (fête), ainsi que des exercices interactifs.</t>
+  </si>
+  <si>
+    <t>Teth (ט) : lettre hébraïque, son et exemples</t>
+  </si>
+  <si>
+    <t>Apprends la lettre hébraïque Teth (ט) et son son [t], son lien avec טוֹב (bon) et des mots comme בֶּטַח (bien sûr), avec des exercices interactifs.</t>
   </si>
   <si>
     <t>Phrases et expressions en hébreu pour débutants</t>
@@ -5367,7 +5385,7 @@
         <v>119</v>
       </c>
       <c r="G22" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H22" t="s">
         <v>30</v>
@@ -7629,7 +7647,7 @@
         <v>370</v>
       </c>
       <c r="G100" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H100" t="s">
         <v>307</v>
@@ -20613,7 +20631,7 @@
         <v>488</v>
       </c>
       <c r="L199" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M199" t="s">
         <v>30</v>
@@ -20675,7 +20693,7 @@
         <v>488</v>
       </c>
       <c r="L200" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M200" t="s">
         <v>307</v>
@@ -20737,7 +20755,7 @@
         <v>488</v>
       </c>
       <c r="L201" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M201" t="s">
         <v>307</v>
@@ -20799,7 +20817,7 @@
         <v>488</v>
       </c>
       <c r="L202" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M202" t="s">
         <v>307</v>
@@ -20861,7 +20879,7 @@
         <v>488</v>
       </c>
       <c r="L203" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M203" t="s">
         <v>307</v>
@@ -20923,7 +20941,7 @@
         <v>488</v>
       </c>
       <c r="L204" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M204" t="s">
         <v>307</v>
@@ -20985,7 +21003,7 @@
         <v>488</v>
       </c>
       <c r="L205" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M205" t="s">
         <v>307</v>
@@ -31959,7 +31977,7 @@
         <v>495</v>
       </c>
       <c r="L382" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M382" t="s">
         <v>307</v>
@@ -38257,7 +38275,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P72"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -39775,7 +39793,7 @@
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>282</v>
+        <v>119</v>
       </c>
       <c r="B31" t="s">
         <v>1286</v>
@@ -39787,10 +39805,10 @@
         <v>1288</v>
       </c>
       <c r="E31" t="s">
-        <v>279</v>
+        <v>116</v>
       </c>
       <c r="F31" t="s">
-        <v>935</v>
+        <v>117</v>
       </c>
       <c r="G31" t="s">
         <v>1289</v>
@@ -39825,7 +39843,7 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>203</v>
+        <v>282</v>
       </c>
       <c r="B32" t="s">
         <v>1290</v>
@@ -39837,10 +39855,10 @@
         <v>1292</v>
       </c>
       <c r="E32" t="s">
-        <v>200</v>
+        <v>279</v>
       </c>
       <c r="F32" t="s">
-        <v>201</v>
+        <v>935</v>
       </c>
       <c r="G32" t="s">
         <v>1293</v>
@@ -39864,7 +39882,7 @@
         <v>2</v>
       </c>
       <c r="N32" t="s">
-        <v>1173</v>
+        <v>1253</v>
       </c>
       <c r="O32" t="s">
         <v>29</v>
@@ -39875,7 +39893,7 @@
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>170</v>
+        <v>203</v>
       </c>
       <c r="B33" t="s">
         <v>1294</v>
@@ -39887,10 +39905,10 @@
         <v>1296</v>
       </c>
       <c r="E33" t="s">
-        <v>167</v>
+        <v>200</v>
       </c>
       <c r="F33" t="s">
-        <v>169</v>
+        <v>201</v>
       </c>
       <c r="G33" t="s">
         <v>1297</v>
@@ -39925,7 +39943,7 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>228</v>
+        <v>170</v>
       </c>
       <c r="B34" t="s">
         <v>1298</v>
@@ -39937,10 +39955,10 @@
         <v>1300</v>
       </c>
       <c r="E34" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="F34" t="s">
-        <v>257</v>
+        <v>169</v>
       </c>
       <c r="G34" t="s">
         <v>1301</v>
@@ -39975,7 +39993,7 @@
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>287</v>
+        <v>228</v>
       </c>
       <c r="B35" t="s">
         <v>1302</v>
@@ -39987,10 +40005,10 @@
         <v>1304</v>
       </c>
       <c r="E35" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F35" t="s">
-        <v>285</v>
+        <v>257</v>
       </c>
       <c r="G35" t="s">
         <v>1305</v>
@@ -40014,7 +40032,7 @@
         <v>2</v>
       </c>
       <c r="N35" t="s">
-        <v>1253</v>
+        <v>1173</v>
       </c>
       <c r="O35" t="s">
         <v>29</v>
@@ -40025,10 +40043,10 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>287</v>
+      </c>
+      <c r="B36" t="s">
         <v>1306</v>
-      </c>
-      <c r="B36" t="s">
-        <v>1307</v>
       </c>
       <c r="C36" t="s">
         <v>1307</v>
@@ -40037,34 +40055,34 @@
         <v>1308</v>
       </c>
       <c r="E36" t="s">
-        <v>2</v>
+        <v>283</v>
       </c>
       <c r="F36" t="s">
-        <v>2</v>
+        <v>285</v>
       </c>
       <c r="G36" t="s">
-        <v>2</v>
+        <v>1309</v>
       </c>
       <c r="H36" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I36" t="s">
-        <v>672</v>
+        <v>2</v>
       </c>
       <c r="J36" t="s">
-        <v>1309</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="L36" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="M36" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N36" t="s">
-        <v>1173</v>
+        <v>1253</v>
       </c>
       <c r="O36" t="s">
         <v>29</v>
@@ -40099,19 +40117,19 @@
         <v>80</v>
       </c>
       <c r="I37" t="s">
-        <v>595</v>
+        <v>672</v>
       </c>
       <c r="J37" t="s">
-        <v>534</v>
+        <v>1313</v>
       </c>
       <c r="K37" t="s">
         <v>80</v>
       </c>
       <c r="L37" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M37" t="s">
-        <v>1313</v>
+        <v>64</v>
       </c>
       <c r="N37" t="s">
         <v>1173</v>
@@ -40146,22 +40164,22 @@
         <v>2</v>
       </c>
       <c r="H38" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="I38" t="s">
-        <v>2</v>
+        <v>595</v>
       </c>
       <c r="J38" t="s">
-        <v>2</v>
+        <v>534</v>
       </c>
       <c r="K38" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="L38" t="s">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="M38" t="s">
-        <v>2</v>
+        <v>1317</v>
       </c>
       <c r="N38" t="s">
         <v>1173</v>
@@ -40175,22 +40193,22 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>302</v>
+        <v>1318</v>
       </c>
       <c r="B39" t="s">
-        <v>1317</v>
+        <v>1319</v>
       </c>
       <c r="C39" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="D39" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="E39" t="s">
-        <v>299</v>
+        <v>2</v>
       </c>
       <c r="F39" t="s">
-        <v>301</v>
+        <v>2</v>
       </c>
       <c r="G39" t="s">
         <v>2</v>
@@ -40214,36 +40232,36 @@
         <v>2</v>
       </c>
       <c r="N39" t="s">
-        <v>2</v>
+        <v>1173</v>
       </c>
       <c r="O39" t="s">
         <v>29</v>
       </c>
       <c r="P39" t="s">
-        <v>959</v>
+        <v>492</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="B40" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="C40" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="D40" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="E40" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="F40" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="G40" t="s">
-        <v>966</v>
+        <v>2</v>
       </c>
       <c r="H40" t="s">
         <v>2</v>
@@ -40275,25 +40293,25 @@
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>322</v>
+        <v>293</v>
       </c>
       <c r="B41" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="C41" t="s">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="D41" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
       <c r="E41" t="s">
-        <v>319</v>
+        <v>288</v>
       </c>
       <c r="F41" t="s">
-        <v>1325</v>
+        <v>290</v>
       </c>
       <c r="G41" t="s">
-        <v>1326</v>
+        <v>966</v>
       </c>
       <c r="H41" t="s">
         <v>2</v>
@@ -40325,7 +40343,7 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B42" t="s">
         <v>1327</v>
@@ -40337,7 +40355,7 @@
         <v>1328</v>
       </c>
       <c r="E42" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="F42" t="s">
         <v>1329</v>
@@ -40375,7 +40393,7 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>349</v>
+        <v>325</v>
       </c>
       <c r="B43" t="s">
         <v>1331</v>
@@ -40387,13 +40405,13 @@
         <v>1332</v>
       </c>
       <c r="E43" t="s">
-        <v>347</v>
+        <v>323</v>
       </c>
       <c r="F43" t="s">
         <v>1333</v>
       </c>
       <c r="G43" t="s">
-        <v>2</v>
+        <v>1334</v>
       </c>
       <c r="H43" t="s">
         <v>2</v>
@@ -40425,25 +40443,25 @@
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="B44" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="C44" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="D44" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="E44" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="F44" t="s">
-        <v>339</v>
+        <v>1337</v>
       </c>
       <c r="G44" t="s">
-        <v>974</v>
+        <v>2</v>
       </c>
       <c r="H44" t="s">
         <v>2</v>
@@ -40475,25 +40493,25 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="B45" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="C45" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="D45" t="s">
-        <v>1337</v>
+        <v>1339</v>
       </c>
       <c r="E45" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="F45" t="s">
-        <v>1338</v>
+        <v>339</v>
       </c>
       <c r="G45" t="s">
-        <v>330</v>
+        <v>974</v>
       </c>
       <c r="H45" t="s">
         <v>2</v>
@@ -40525,25 +40543,25 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B46" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="C46" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="D46" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="E46" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="F46" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="G46" t="s">
-        <v>1342</v>
+        <v>330</v>
       </c>
       <c r="H46" t="s">
         <v>2</v>
@@ -40575,7 +40593,7 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="B47" t="s">
         <v>1343</v>
@@ -40587,13 +40605,13 @@
         <v>1344</v>
       </c>
       <c r="E47" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="F47" t="s">
-        <v>333</v>
+        <v>1345</v>
       </c>
       <c r="G47" t="s">
-        <v>2</v>
+        <v>1346</v>
       </c>
       <c r="H47" t="s">
         <v>2</v>
@@ -40625,22 +40643,22 @@
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>352</v>
+        <v>334</v>
       </c>
       <c r="B48" t="s">
-        <v>1345</v>
+        <v>1347</v>
       </c>
       <c r="C48" t="s">
-        <v>1345</v>
+        <v>1347</v>
       </c>
       <c r="D48" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
       <c r="E48" t="s">
-        <v>350</v>
+        <v>332</v>
       </c>
       <c r="F48" t="s">
-        <v>351</v>
+        <v>333</v>
       </c>
       <c r="G48" t="s">
         <v>2</v>
@@ -40675,25 +40693,25 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>375</v>
+        <v>352</v>
       </c>
       <c r="B49" t="s">
-        <v>1347</v>
+        <v>1349</v>
       </c>
       <c r="C49" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="D49" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="E49" t="s">
-        <v>371</v>
+        <v>350</v>
       </c>
       <c r="F49" t="s">
-        <v>373</v>
+        <v>351</v>
       </c>
       <c r="G49" t="s">
-        <v>1350</v>
+        <v>2</v>
       </c>
       <c r="H49" t="s">
         <v>2</v>
@@ -40725,7 +40743,7 @@
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>298</v>
+        <v>370</v>
       </c>
       <c r="B50" t="s">
         <v>1351</v>
@@ -40737,13 +40755,13 @@
         <v>1352</v>
       </c>
       <c r="E50" t="s">
-        <v>294</v>
+        <v>368</v>
       </c>
       <c r="F50" t="s">
-        <v>296</v>
+        <v>369</v>
       </c>
       <c r="G50" t="s">
-        <v>1353</v>
+        <v>2</v>
       </c>
       <c r="H50" t="s">
         <v>2</v>
@@ -40775,10 +40793,10 @@
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B51" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="C51" t="s">
         <v>1354</v>
@@ -40787,13 +40805,13 @@
         <v>1355</v>
       </c>
       <c r="E51" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="F51" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="G51" t="s">
-        <v>988</v>
+        <v>1356</v>
       </c>
       <c r="H51" t="s">
         <v>2</v>
@@ -40825,25 +40843,25 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>385</v>
+        <v>298</v>
       </c>
       <c r="B52" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="C52" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="D52" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="E52" t="s">
-        <v>381</v>
+        <v>294</v>
       </c>
       <c r="F52" t="s">
-        <v>383</v>
+        <v>296</v>
       </c>
       <c r="G52" t="s">
-        <v>2</v>
+        <v>1359</v>
       </c>
       <c r="H52" t="s">
         <v>2</v>
@@ -40875,25 +40893,25 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
       <c r="B53" t="s">
-        <v>1358</v>
+        <v>1360</v>
       </c>
       <c r="C53" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="D53" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="E53" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="F53" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="G53" t="s">
-        <v>2</v>
+        <v>988</v>
       </c>
       <c r="H53" t="s">
         <v>2</v>
@@ -40925,25 +40943,25 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="B54" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="C54" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="D54" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="E54" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="F54" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="G54" t="s">
-        <v>995</v>
+        <v>2</v>
       </c>
       <c r="H54" t="s">
         <v>2</v>
@@ -40975,25 +40993,25 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="B55" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="C55" t="s">
-        <v>1363</v>
+        <v>1365</v>
       </c>
       <c r="D55" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="E55" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="F55" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="G55" t="s">
-        <v>1365</v>
+        <v>2</v>
       </c>
       <c r="H55" t="s">
         <v>2</v>
@@ -41025,25 +41043,25 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
       <c r="B56" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="C56" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="D56" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="E56" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="F56" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="G56" t="s">
-        <v>1368</v>
+        <v>995</v>
       </c>
       <c r="H56" t="s">
         <v>2</v>
@@ -41075,7 +41093,7 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
       <c r="B57" t="s">
         <v>1369</v>
@@ -41087,10 +41105,10 @@
         <v>1370</v>
       </c>
       <c r="E57" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="F57" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="G57" t="s">
         <v>1371</v>
@@ -41125,7 +41143,7 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
       <c r="B58" t="s">
         <v>1372</v>
@@ -41137,13 +41155,13 @@
         <v>1373</v>
       </c>
       <c r="E58" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="F58" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="G58" t="s">
-        <v>1016</v>
+        <v>1374</v>
       </c>
       <c r="H58" t="s">
         <v>2</v>
@@ -41175,25 +41193,25 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="B59" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="C59" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="D59" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="E59" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="F59" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="G59" t="s">
-        <v>1019</v>
+        <v>1377</v>
       </c>
       <c r="H59" t="s">
         <v>2</v>
@@ -41225,25 +41243,25 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="B60" t="s">
-        <v>1376</v>
+        <v>1378</v>
       </c>
       <c r="C60" t="s">
-        <v>1376</v>
+        <v>1378</v>
       </c>
       <c r="D60" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="E60" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="F60" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="G60" t="s">
-        <v>1378</v>
+        <v>1016</v>
       </c>
       <c r="H60" t="s">
         <v>2</v>
@@ -41275,25 +41293,25 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="B61" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
       <c r="C61" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
       <c r="D61" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="E61" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="F61" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="G61" t="s">
-        <v>1027</v>
+        <v>1019</v>
       </c>
       <c r="H61" t="s">
         <v>2</v>
@@ -41325,25 +41343,25 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="B62" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="C62" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="D62" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="E62" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="F62" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="G62" t="s">
-        <v>1031</v>
+        <v>1384</v>
       </c>
       <c r="H62" t="s">
         <v>2</v>
@@ -41375,25 +41393,25 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="B63" t="s">
-        <v>1383</v>
+        <v>1385</v>
       </c>
       <c r="C63" t="s">
-        <v>1383</v>
+        <v>1385</v>
       </c>
       <c r="D63" t="s">
-        <v>1384</v>
+        <v>1386</v>
       </c>
       <c r="E63" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="F63" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="G63" t="s">
-        <v>1031</v>
+        <v>1027</v>
       </c>
       <c r="H63" t="s">
         <v>2</v>
@@ -41425,25 +41443,25 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
       <c r="B64" t="s">
-        <v>1385</v>
+        <v>1387</v>
       </c>
       <c r="C64" t="s">
-        <v>1385</v>
+        <v>1387</v>
       </c>
       <c r="D64" t="s">
-        <v>1386</v>
+        <v>1388</v>
       </c>
       <c r="E64" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="F64" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="G64" t="s">
-        <v>1037</v>
+        <v>1031</v>
       </c>
       <c r="H64" t="s">
         <v>2</v>
@@ -41475,25 +41493,25 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>438</v>
+        <v>430</v>
       </c>
       <c r="B65" t="s">
-        <v>1387</v>
+        <v>1389</v>
       </c>
       <c r="C65" t="s">
-        <v>1387</v>
+        <v>1389</v>
       </c>
       <c r="D65" t="s">
-        <v>1388</v>
+        <v>1390</v>
       </c>
       <c r="E65" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="F65" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="G65" t="s">
-        <v>1040</v>
+        <v>1031</v>
       </c>
       <c r="H65" t="s">
         <v>2</v>
@@ -41525,25 +41543,25 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>442</v>
+        <v>434</v>
       </c>
       <c r="B66" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
       <c r="C66" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
       <c r="D66" t="s">
-        <v>1390</v>
+        <v>1392</v>
       </c>
       <c r="E66" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
       <c r="F66" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="G66" t="s">
-        <v>1044</v>
+        <v>1037</v>
       </c>
       <c r="H66" t="s">
         <v>2</v>
@@ -41575,25 +41593,25 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
       <c r="B67" t="s">
-        <v>1391</v>
+        <v>1393</v>
       </c>
       <c r="C67" t="s">
-        <v>1392</v>
+        <v>1393</v>
       </c>
       <c r="D67" t="s">
-        <v>1393</v>
+        <v>1394</v>
       </c>
       <c r="E67" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="F67" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="G67" t="s">
-        <v>1047</v>
+        <v>1040</v>
       </c>
       <c r="H67" t="s">
         <v>2</v>
@@ -41625,10 +41643,10 @@
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="B68" t="s">
-        <v>1394</v>
+        <v>1395</v>
       </c>
       <c r="C68" t="s">
         <v>1395</v>
@@ -41637,13 +41655,13 @@
         <v>1396</v>
       </c>
       <c r="E68" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="F68" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
       <c r="G68" t="s">
-        <v>1397</v>
+        <v>1044</v>
       </c>
       <c r="H68" t="s">
         <v>2</v>
@@ -41664,36 +41682,36 @@
         <v>2</v>
       </c>
       <c r="N68" t="s">
-        <v>1253</v>
+        <v>2</v>
       </c>
       <c r="O68" t="s">
         <v>29</v>
       </c>
       <c r="P68" t="s">
-        <v>492</v>
+        <v>959</v>
       </c>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>461</v>
+        <v>446</v>
       </c>
       <c r="B69" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C69" t="s">
         <v>1398</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>1399</v>
       </c>
-      <c r="D69" t="s">
-        <v>1400</v>
-      </c>
       <c r="E69" t="s">
-        <v>457</v>
+        <v>443</v>
       </c>
       <c r="F69" t="s">
-        <v>459</v>
+        <v>445</v>
       </c>
       <c r="G69" t="s">
-        <v>1401</v>
+        <v>1047</v>
       </c>
       <c r="H69" t="s">
         <v>2</v>
@@ -41714,36 +41732,36 @@
         <v>2</v>
       </c>
       <c r="N69" t="s">
-        <v>1253</v>
+        <v>2</v>
       </c>
       <c r="O69" t="s">
         <v>29</v>
       </c>
       <c r="P69" t="s">
-        <v>492</v>
+        <v>959</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>466</v>
+        <v>450</v>
       </c>
       <c r="B70" t="s">
+        <v>1400</v>
+      </c>
+      <c r="C70" t="s">
+        <v>1401</v>
+      </c>
+      <c r="D70" t="s">
         <v>1402</v>
       </c>
-      <c r="C70" t="s">
+      <c r="E70" t="s">
+        <v>447</v>
+      </c>
+      <c r="F70" t="s">
+        <v>449</v>
+      </c>
+      <c r="G70" t="s">
         <v>1403</v>
-      </c>
-      <c r="D70" t="s">
-        <v>1404</v>
-      </c>
-      <c r="E70" t="s">
-        <v>463</v>
-      </c>
-      <c r="F70" t="s">
-        <v>465</v>
-      </c>
-      <c r="G70" t="s">
-        <v>1405</v>
       </c>
       <c r="H70" t="s">
         <v>2</v>
@@ -41770,6 +41788,106 @@
         <v>29</v>
       </c>
       <c r="P70" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>461</v>
+      </c>
+      <c r="B71" t="s">
+        <v>1404</v>
+      </c>
+      <c r="C71" t="s">
+        <v>1405</v>
+      </c>
+      <c r="D71" t="s">
+        <v>1406</v>
+      </c>
+      <c r="E71" t="s">
+        <v>457</v>
+      </c>
+      <c r="F71" t="s">
+        <v>459</v>
+      </c>
+      <c r="G71" t="s">
+        <v>1407</v>
+      </c>
+      <c r="H71" t="s">
+        <v>2</v>
+      </c>
+      <c r="I71" t="s">
+        <v>2</v>
+      </c>
+      <c r="J71" t="s">
+        <v>2</v>
+      </c>
+      <c r="K71" t="s">
+        <v>2</v>
+      </c>
+      <c r="L71" t="s">
+        <v>2</v>
+      </c>
+      <c r="M71" t="s">
+        <v>2</v>
+      </c>
+      <c r="N71" t="s">
+        <v>1253</v>
+      </c>
+      <c r="O71" t="s">
+        <v>29</v>
+      </c>
+      <c r="P71" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>466</v>
+      </c>
+      <c r="B72" t="s">
+        <v>1408</v>
+      </c>
+      <c r="C72" t="s">
+        <v>1409</v>
+      </c>
+      <c r="D72" t="s">
+        <v>1410</v>
+      </c>
+      <c r="E72" t="s">
+        <v>463</v>
+      </c>
+      <c r="F72" t="s">
+        <v>465</v>
+      </c>
+      <c r="G72" t="s">
+        <v>1411</v>
+      </c>
+      <c r="H72" t="s">
+        <v>2</v>
+      </c>
+      <c r="I72" t="s">
+        <v>2</v>
+      </c>
+      <c r="J72" t="s">
+        <v>2</v>
+      </c>
+      <c r="K72" t="s">
+        <v>2</v>
+      </c>
+      <c r="L72" t="s">
+        <v>2</v>
+      </c>
+      <c r="M72" t="s">
+        <v>2</v>
+      </c>
+      <c r="N72" t="s">
+        <v>1253</v>
+      </c>
+      <c r="O72" t="s">
+        <v>29</v>
+      </c>
+      <c r="P72" t="s">
         <v>492</v>
       </c>
     </row>
@@ -41782,7 +41900,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -41809,7 +41927,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1406</v>
+        <v>1412</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -42024,22 +42142,22 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="B11" t="s">
         <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="D11" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="E11" t="s">
         <v>37</v>
       </c>
       <c r="F11">
-        <v>17.4</v>
+        <v>16</v>
       </c>
       <c r="G11" t="s">
         <v>30</v>
@@ -42047,22 +42165,22 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
       <c r="E12" t="s">
         <v>37</v>
       </c>
       <c r="F12">
-        <v>16</v>
+        <v>13.9</v>
       </c>
       <c r="G12" t="s">
         <v>30</v>
@@ -42070,16 +42188,16 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D13" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E13" t="s">
         <v>37</v>
@@ -42093,22 +42211,22 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>121</v>
       </c>
       <c r="D14" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="E14" t="s">
         <v>37</v>
       </c>
       <c r="F14">
-        <v>13.9</v>
+        <v>12.3</v>
       </c>
       <c r="G14" t="s">
         <v>30</v>
@@ -42116,19 +42234,19 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>120</v>
+        <v>283</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>284</v>
       </c>
       <c r="C15" t="s">
-        <v>121</v>
+        <v>285</v>
       </c>
       <c r="D15" t="s">
-        <v>123</v>
+        <v>287</v>
       </c>
       <c r="E15" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F15">
         <v>12.3</v>
@@ -42139,22 +42257,22 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>283</v>
+        <v>154</v>
       </c>
       <c r="B16" t="s">
-        <v>284</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>285</v>
+        <v>155</v>
       </c>
       <c r="D16" t="s">
-        <v>287</v>
+        <v>157</v>
       </c>
       <c r="E16" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F16">
-        <v>12.3</v>
+        <v>10.3</v>
       </c>
       <c r="G16" t="s">
         <v>30</v>
@@ -42162,16 +42280,16 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>154</v>
+        <v>303</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>304</v>
       </c>
       <c r="C17" t="s">
-        <v>155</v>
+        <v>305</v>
       </c>
       <c r="D17" t="s">
-        <v>157</v>
+        <v>306</v>
       </c>
       <c r="E17" t="s">
         <v>37</v>
@@ -42180,24 +42298,24 @@
         <v>10.3</v>
       </c>
       <c r="G17" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>303</v>
+        <v>447</v>
       </c>
       <c r="B18" t="s">
-        <v>304</v>
+        <v>448</v>
       </c>
       <c r="C18" t="s">
-        <v>305</v>
+        <v>449</v>
       </c>
       <c r="D18" t="s">
-        <v>306</v>
+        <v>450</v>
       </c>
       <c r="E18" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F18">
         <v>10.3</v>
@@ -42208,68 +42326,68 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>447</v>
+        <v>273</v>
       </c>
       <c r="B19" t="s">
-        <v>448</v>
+        <v>274</v>
       </c>
       <c r="C19" t="s">
-        <v>449</v>
+        <v>275</v>
       </c>
       <c r="D19" t="s">
-        <v>450</v>
+        <v>143</v>
       </c>
       <c r="E19" t="s">
         <v>183</v>
       </c>
       <c r="F19">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="G19" t="s">
-        <v>307</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>273</v>
+        <v>308</v>
       </c>
       <c r="B20" t="s">
-        <v>274</v>
+        <v>304</v>
       </c>
       <c r="C20" t="s">
-        <v>275</v>
+        <v>309</v>
       </c>
       <c r="D20" t="s">
-        <v>143</v>
+        <v>311</v>
       </c>
       <c r="E20" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F20">
-        <v>10</v>
+        <v>9.8</v>
       </c>
       <c r="G20" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="B21" t="s">
         <v>304</v>
       </c>
       <c r="C21" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D21" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="E21" t="s">
         <v>37</v>
       </c>
       <c r="F21">
-        <v>9.8</v>
+        <v>9.3</v>
       </c>
       <c r="G21" t="s">
         <v>307</v>
@@ -42277,16 +42395,16 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B22" t="s">
         <v>304</v>
       </c>
       <c r="C22" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="D22" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="E22" t="s">
         <v>37</v>
@@ -42300,45 +42418,45 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>316</v>
+        <v>158</v>
       </c>
       <c r="B23" t="s">
-        <v>304</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>317</v>
+        <v>159</v>
       </c>
       <c r="D23" t="s">
-        <v>318</v>
+        <v>161</v>
       </c>
       <c r="E23" t="s">
         <v>37</v>
       </c>
       <c r="F23">
-        <v>9.3</v>
+        <v>9</v>
       </c>
       <c r="G23" t="s">
-        <v>307</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>180</v>
       </c>
       <c r="C24" t="s">
-        <v>159</v>
+        <v>181</v>
       </c>
       <c r="D24" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="E24" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F24">
-        <v>9</v>
+        <v>8.3</v>
       </c>
       <c r="G24" t="s">
         <v>30</v>
@@ -42346,39 +42464,39 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>179</v>
+        <v>335</v>
       </c>
       <c r="B25" t="s">
-        <v>180</v>
+        <v>304</v>
       </c>
       <c r="C25" t="s">
-        <v>181</v>
+        <v>336</v>
       </c>
       <c r="D25" t="s">
-        <v>182</v>
+        <v>337</v>
       </c>
       <c r="E25" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F25">
         <v>8.3</v>
       </c>
       <c r="G25" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="B26" t="s">
         <v>304</v>
       </c>
       <c r="C26" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="D26" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="E26" t="s">
         <v>37</v>
@@ -42392,16 +42510,16 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B27" t="s">
         <v>304</v>
       </c>
       <c r="C27" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D27" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="E27" t="s">
         <v>37</v>
@@ -42415,39 +42533,39 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>344</v>
+        <v>267</v>
       </c>
       <c r="B28" t="s">
-        <v>304</v>
+        <v>268</v>
       </c>
       <c r="C28" t="s">
-        <v>345</v>
+        <v>269</v>
       </c>
       <c r="D28" t="s">
-        <v>346</v>
+        <v>193</v>
       </c>
       <c r="E28" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F28">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G28" t="s">
-        <v>307</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B29" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C29" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D29" t="s">
-        <v>193</v>
+        <v>247</v>
       </c>
       <c r="E29" t="s">
         <v>183</v>
@@ -42461,39 +42579,39 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>270</v>
+        <v>353</v>
       </c>
       <c r="B30" t="s">
-        <v>271</v>
+        <v>304</v>
       </c>
       <c r="C30" t="s">
-        <v>272</v>
+        <v>354</v>
       </c>
       <c r="D30" t="s">
-        <v>247</v>
+        <v>355</v>
       </c>
       <c r="E30" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F30">
         <v>8</v>
       </c>
       <c r="G30" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B31" t="s">
         <v>304</v>
       </c>
       <c r="C31" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D31" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="E31" t="s">
         <v>37</v>
@@ -42507,16 +42625,16 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B32" t="s">
         <v>304</v>
       </c>
       <c r="C32" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D32" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="E32" t="s">
         <v>37</v>
@@ -42530,16 +42648,16 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B33" t="s">
         <v>304</v>
       </c>
       <c r="C33" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="D33" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E33" t="s">
         <v>37</v>
@@ -42553,16 +42671,16 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B34" t="s">
         <v>304</v>
       </c>
       <c r="C34" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="D34" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="E34" t="s">
         <v>37</v>
@@ -42576,70 +42694,24 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>365</v>
+        <v>276</v>
       </c>
       <c r="B35" t="s">
-        <v>304</v>
+        <v>277</v>
       </c>
       <c r="C35" t="s">
-        <v>366</v>
+        <v>278</v>
       </c>
       <c r="D35" t="s">
-        <v>367</v>
+        <v>2</v>
       </c>
       <c r="E35" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F35">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="G35" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>368</v>
-      </c>
-      <c r="B36" t="s">
-        <v>304</v>
-      </c>
-      <c r="C36" t="s">
-        <v>369</v>
-      </c>
-      <c r="D36" t="s">
-        <v>370</v>
-      </c>
-      <c r="E36" t="s">
-        <v>37</v>
-      </c>
-      <c r="F36">
-        <v>8</v>
-      </c>
-      <c r="G36" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>276</v>
-      </c>
-      <c r="B37" t="s">
-        <v>277</v>
-      </c>
-      <c r="C37" t="s">
-        <v>278</v>
-      </c>
-      <c r="D37" t="s">
-        <v>2</v>
-      </c>
-      <c r="E37" t="s">
-        <v>183</v>
-      </c>
-      <c r="F37">
-        <v>0.8</v>
-      </c>
-      <c r="G37" t="s">
         <v>30</v>
       </c>
     </row>
@@ -42746,27 +42818,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>1407</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1408</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1409</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1410</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1411</v>
+        <v>1417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Yod letter lesson (EN + FR)
Normalizes the tenth letter lesson from its pinned raw snapshots in both
locales, no holdouts. Editorial review: "final Dalet/Yud" becomes "at the
end of the word" in both locales, FR "ch" -> "kh" for חַי, FR
"Conclusions" -> "À retenir", and (owner decisions) the intro compares
Yod to a short Vav, the dot in בִּי is named Hiriq, and the SEO spelling
Yod is used with "also spelled Yud" once (new general rule). Registers
SEO (EN and FR clusters and keywords planned -> published, pages rows),
links it from the alphabet guide, and publishes both locales on
2026-10-26.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seo/semantic-core.xlsx
+++ b/docs/seo/semantic-core.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12162" uniqueCount="1418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12182" uniqueCount="1424">
   <si>
     <t>HebrewEdu Semantic Core — generated view</t>
   </si>
@@ -3889,6 +3889,18 @@
     <t>hebrew tet pronunciation; hebrew letter tet sound; learn hebrew letter tet; tet hebrew letter exercises; teth hebrew letter; tet vs tav hebrew pronunciation</t>
   </si>
   <si>
+    <t>Yod Hebrew Letter (י): Sound &amp; Words</t>
+  </si>
+  <si>
+    <t>Yod Hebrew Letter (י): Sound, Words &amp; Practice</t>
+  </si>
+  <si>
+    <t>Learn the Hebrew letter Yod (י), also spelled Yud: its [y] sound, how it helps spell the vowel [i], words like יָד (hand), plus interactive practice.</t>
+  </si>
+  <si>
+    <t>yud hebrew letter; hebrew yod pronunciation; hebrew letter yod sound; learn hebrew letter yod; yod hebrew letter exercises; yod with hiriq; yod vs vav hebrew letters</t>
+  </si>
+  <si>
     <t>Hebrew Phrases for Beginners: 30 Useful Phrases</t>
   </si>
   <si>
@@ -4076,6 +4088,12 @@
   </si>
   <si>
     <t>Apprends la lettre hébraïque Teth (ט) et son son [t], son lien avec טוֹב (bon) et des mots comme בֶּטַח (bien sûr), avec des exercices interactifs.</t>
+  </si>
+  <si>
+    <t>Yod (י) : lettre hébraïque, son et exemples</t>
+  </si>
+  <si>
+    <t>Apprends la lettre hébraïque Yod (י) : son son [y], son rôle pour noter la voyelle [i] et des mots comme יָד (main), avec des exercices interactifs.</t>
   </si>
   <si>
     <t>Phrases et expressions en hébreu pour débutants</t>
@@ -5008,7 +5026,7 @@
         <v>65</v>
       </c>
       <c r="G9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H9" t="s">
         <v>30</v>
@@ -7154,7 +7172,7 @@
         <v>318</v>
       </c>
       <c r="G83" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H83" t="s">
         <v>307</v>
@@ -21065,7 +21083,7 @@
         <v>488</v>
       </c>
       <c r="L206" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M206" t="s">
         <v>30</v>
@@ -21127,7 +21145,7 @@
         <v>488</v>
       </c>
       <c r="L207" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M207" t="s">
         <v>307</v>
@@ -21189,7 +21207,7 @@
         <v>488</v>
       </c>
       <c r="L208" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M208" t="s">
         <v>307</v>
@@ -21251,7 +21269,7 @@
         <v>488</v>
       </c>
       <c r="L209" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M209" t="s">
         <v>307</v>
@@ -21313,7 +21331,7 @@
         <v>488</v>
       </c>
       <c r="L210" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M210" t="s">
         <v>307</v>
@@ -21375,7 +21393,7 @@
         <v>488</v>
       </c>
       <c r="L211" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M211" t="s">
         <v>307</v>
@@ -21437,7 +21455,7 @@
         <v>488</v>
       </c>
       <c r="L212" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M212" t="s">
         <v>307</v>
@@ -21499,7 +21517,7 @@
         <v>488</v>
       </c>
       <c r="L213" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M213" t="s">
         <v>307</v>
@@ -30923,7 +30941,7 @@
         <v>495</v>
       </c>
       <c r="L365" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M365" t="s">
         <v>307</v>
@@ -38275,7 +38293,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P72"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
@@ -39843,7 +39861,7 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>282</v>
+        <v>65</v>
       </c>
       <c r="B32" t="s">
         <v>1290</v>
@@ -39855,10 +39873,10 @@
         <v>1292</v>
       </c>
       <c r="E32" t="s">
-        <v>279</v>
+        <v>61</v>
       </c>
       <c r="F32" t="s">
-        <v>935</v>
+        <v>62</v>
       </c>
       <c r="G32" t="s">
         <v>1293</v>
@@ -39893,7 +39911,7 @@
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>203</v>
+        <v>282</v>
       </c>
       <c r="B33" t="s">
         <v>1294</v>
@@ -39905,10 +39923,10 @@
         <v>1296</v>
       </c>
       <c r="E33" t="s">
-        <v>200</v>
+        <v>279</v>
       </c>
       <c r="F33" t="s">
-        <v>201</v>
+        <v>935</v>
       </c>
       <c r="G33" t="s">
         <v>1297</v>
@@ -39932,7 +39950,7 @@
         <v>2</v>
       </c>
       <c r="N33" t="s">
-        <v>1173</v>
+        <v>1253</v>
       </c>
       <c r="O33" t="s">
         <v>29</v>
@@ -39943,7 +39961,7 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>170</v>
+        <v>203</v>
       </c>
       <c r="B34" t="s">
         <v>1298</v>
@@ -39955,10 +39973,10 @@
         <v>1300</v>
       </c>
       <c r="E34" t="s">
-        <v>167</v>
+        <v>200</v>
       </c>
       <c r="F34" t="s">
-        <v>169</v>
+        <v>201</v>
       </c>
       <c r="G34" t="s">
         <v>1301</v>
@@ -39993,7 +40011,7 @@
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>228</v>
+        <v>170</v>
       </c>
       <c r="B35" t="s">
         <v>1302</v>
@@ -40005,10 +40023,10 @@
         <v>1304</v>
       </c>
       <c r="E35" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="F35" t="s">
-        <v>257</v>
+        <v>169</v>
       </c>
       <c r="G35" t="s">
         <v>1305</v>
@@ -40043,7 +40061,7 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>287</v>
+        <v>228</v>
       </c>
       <c r="B36" t="s">
         <v>1306</v>
@@ -40055,10 +40073,10 @@
         <v>1308</v>
       </c>
       <c r="E36" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F36" t="s">
-        <v>285</v>
+        <v>257</v>
       </c>
       <c r="G36" t="s">
         <v>1309</v>
@@ -40082,7 +40100,7 @@
         <v>2</v>
       </c>
       <c r="N36" t="s">
-        <v>1253</v>
+        <v>1173</v>
       </c>
       <c r="O36" t="s">
         <v>29</v>
@@ -40093,10 +40111,10 @@
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B37" t="s">
         <v>1310</v>
-      </c>
-      <c r="B37" t="s">
-        <v>1311</v>
       </c>
       <c r="C37" t="s">
         <v>1311</v>
@@ -40105,34 +40123,34 @@
         <v>1312</v>
       </c>
       <c r="E37" t="s">
-        <v>2</v>
+        <v>283</v>
       </c>
       <c r="F37" t="s">
-        <v>2</v>
+        <v>285</v>
       </c>
       <c r="G37" t="s">
-        <v>2</v>
+        <v>1313</v>
       </c>
       <c r="H37" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I37" t="s">
-        <v>672</v>
+        <v>2</v>
       </c>
       <c r="J37" t="s">
-        <v>1313</v>
+        <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="L37" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="M37" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N37" t="s">
-        <v>1173</v>
+        <v>1253</v>
       </c>
       <c r="O37" t="s">
         <v>29</v>
@@ -40167,19 +40185,19 @@
         <v>80</v>
       </c>
       <c r="I38" t="s">
-        <v>595</v>
+        <v>672</v>
       </c>
       <c r="J38" t="s">
-        <v>534</v>
+        <v>1317</v>
       </c>
       <c r="K38" t="s">
         <v>80</v>
       </c>
       <c r="L38" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="M38" t="s">
-        <v>1317</v>
+        <v>64</v>
       </c>
       <c r="N38" t="s">
         <v>1173</v>
@@ -40214,22 +40232,22 @@
         <v>2</v>
       </c>
       <c r="H39" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="I39" t="s">
-        <v>2</v>
+        <v>595</v>
       </c>
       <c r="J39" t="s">
-        <v>2</v>
+        <v>534</v>
       </c>
       <c r="K39" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="L39" t="s">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="M39" t="s">
-        <v>2</v>
+        <v>1321</v>
       </c>
       <c r="N39" t="s">
         <v>1173</v>
@@ -40243,22 +40261,22 @@
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>302</v>
+        <v>1322</v>
       </c>
       <c r="B40" t="s">
-        <v>1321</v>
+        <v>1323</v>
       </c>
       <c r="C40" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="D40" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="E40" t="s">
-        <v>299</v>
+        <v>2</v>
       </c>
       <c r="F40" t="s">
-        <v>301</v>
+        <v>2</v>
       </c>
       <c r="G40" t="s">
         <v>2</v>
@@ -40282,36 +40300,36 @@
         <v>2</v>
       </c>
       <c r="N40" t="s">
-        <v>2</v>
+        <v>1173</v>
       </c>
       <c r="O40" t="s">
         <v>29</v>
       </c>
       <c r="P40" t="s">
-        <v>959</v>
+        <v>492</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="B41" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="C41" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="D41" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="E41" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="F41" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="G41" t="s">
-        <v>966</v>
+        <v>2</v>
       </c>
       <c r="H41" t="s">
         <v>2</v>
@@ -40343,25 +40361,25 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>322</v>
+        <v>293</v>
       </c>
       <c r="B42" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="C42" t="s">
-        <v>1327</v>
+        <v>1329</v>
       </c>
       <c r="D42" t="s">
-        <v>1328</v>
+        <v>1330</v>
       </c>
       <c r="E42" t="s">
-        <v>319</v>
+        <v>288</v>
       </c>
       <c r="F42" t="s">
-        <v>1329</v>
+        <v>290</v>
       </c>
       <c r="G42" t="s">
-        <v>1330</v>
+        <v>966</v>
       </c>
       <c r="H42" t="s">
         <v>2</v>
@@ -40393,7 +40411,7 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B43" t="s">
         <v>1331</v>
@@ -40405,7 +40423,7 @@
         <v>1332</v>
       </c>
       <c r="E43" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="F43" t="s">
         <v>1333</v>
@@ -40443,7 +40461,7 @@
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>349</v>
+        <v>325</v>
       </c>
       <c r="B44" t="s">
         <v>1335</v>
@@ -40455,13 +40473,13 @@
         <v>1336</v>
       </c>
       <c r="E44" t="s">
-        <v>347</v>
+        <v>323</v>
       </c>
       <c r="F44" t="s">
         <v>1337</v>
       </c>
       <c r="G44" t="s">
-        <v>2</v>
+        <v>1338</v>
       </c>
       <c r="H44" t="s">
         <v>2</v>
@@ -40493,25 +40511,25 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="B45" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="C45" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="D45" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="E45" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="F45" t="s">
-        <v>339</v>
+        <v>1341</v>
       </c>
       <c r="G45" t="s">
-        <v>974</v>
+        <v>2</v>
       </c>
       <c r="H45" t="s">
         <v>2</v>
@@ -40543,25 +40561,25 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="B46" t="s">
-        <v>1340</v>
+        <v>1342</v>
       </c>
       <c r="C46" t="s">
-        <v>1340</v>
+        <v>1342</v>
       </c>
       <c r="D46" t="s">
-        <v>1341</v>
+        <v>1343</v>
       </c>
       <c r="E46" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="F46" t="s">
-        <v>1342</v>
+        <v>339</v>
       </c>
       <c r="G46" t="s">
-        <v>330</v>
+        <v>974</v>
       </c>
       <c r="H46" t="s">
         <v>2</v>
@@ -40593,25 +40611,25 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B47" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="C47" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="D47" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="E47" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="F47" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="G47" t="s">
-        <v>1346</v>
+        <v>330</v>
       </c>
       <c r="H47" t="s">
         <v>2</v>
@@ -40643,7 +40661,7 @@
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="B48" t="s">
         <v>1347</v>
@@ -40655,13 +40673,13 @@
         <v>1348</v>
       </c>
       <c r="E48" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="F48" t="s">
-        <v>333</v>
+        <v>1349</v>
       </c>
       <c r="G48" t="s">
-        <v>2</v>
+        <v>1350</v>
       </c>
       <c r="H48" t="s">
         <v>2</v>
@@ -40693,22 +40711,22 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>352</v>
+        <v>334</v>
       </c>
       <c r="B49" t="s">
-        <v>1349</v>
+        <v>1351</v>
       </c>
       <c r="C49" t="s">
-        <v>1349</v>
+        <v>1351</v>
       </c>
       <c r="D49" t="s">
-        <v>1350</v>
+        <v>1352</v>
       </c>
       <c r="E49" t="s">
-        <v>350</v>
+        <v>332</v>
       </c>
       <c r="F49" t="s">
-        <v>351</v>
+        <v>333</v>
       </c>
       <c r="G49" t="s">
         <v>2</v>
@@ -40743,22 +40761,22 @@
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>370</v>
+        <v>352</v>
       </c>
       <c r="B50" t="s">
-        <v>1351</v>
+        <v>1353</v>
       </c>
       <c r="C50" t="s">
-        <v>1351</v>
+        <v>1353</v>
       </c>
       <c r="D50" t="s">
-        <v>1352</v>
+        <v>1354</v>
       </c>
       <c r="E50" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="F50" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
       <c r="G50" t="s">
         <v>2</v>
@@ -40793,25 +40811,25 @@
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B51" t="s">
-        <v>1353</v>
+        <v>1355</v>
       </c>
       <c r="C51" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="D51" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="E51" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="F51" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="G51" t="s">
-        <v>1356</v>
+        <v>2</v>
       </c>
       <c r="H51" t="s">
         <v>2</v>
@@ -40843,7 +40861,7 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>298</v>
+        <v>318</v>
       </c>
       <c r="B52" t="s">
         <v>1357</v>
@@ -40855,13 +40873,13 @@
         <v>1358</v>
       </c>
       <c r="E52" t="s">
-        <v>294</v>
+        <v>316</v>
       </c>
       <c r="F52" t="s">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="G52" t="s">
-        <v>1359</v>
+        <v>2</v>
       </c>
       <c r="H52" t="s">
         <v>2</v>
@@ -40893,10 +40911,10 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B53" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="C53" t="s">
         <v>1360</v>
@@ -40905,13 +40923,13 @@
         <v>1361</v>
       </c>
       <c r="E53" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="F53" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="G53" t="s">
-        <v>988</v>
+        <v>1362</v>
       </c>
       <c r="H53" t="s">
         <v>2</v>
@@ -40943,25 +40961,25 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>385</v>
+        <v>298</v>
       </c>
       <c r="B54" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="C54" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="D54" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="E54" t="s">
-        <v>381</v>
+        <v>294</v>
       </c>
       <c r="F54" t="s">
-        <v>383</v>
+        <v>296</v>
       </c>
       <c r="G54" t="s">
-        <v>2</v>
+        <v>1365</v>
       </c>
       <c r="H54" t="s">
         <v>2</v>
@@ -40993,25 +41011,25 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
       <c r="B55" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="C55" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="D55" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="E55" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="F55" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="G55" t="s">
-        <v>2</v>
+        <v>988</v>
       </c>
       <c r="H55" t="s">
         <v>2</v>
@@ -41043,25 +41061,25 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="B56" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="C56" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="D56" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="E56" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="F56" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="G56" t="s">
-        <v>995</v>
+        <v>2</v>
       </c>
       <c r="H56" t="s">
         <v>2</v>
@@ -41093,25 +41111,25 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="B57" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="C57" t="s">
-        <v>1369</v>
+        <v>1371</v>
       </c>
       <c r="D57" t="s">
-        <v>1370</v>
+        <v>1372</v>
       </c>
       <c r="E57" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="F57" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="G57" t="s">
-        <v>1371</v>
+        <v>2</v>
       </c>
       <c r="H57" t="s">
         <v>2</v>
@@ -41143,25 +41161,25 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
       <c r="B58" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="C58" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="D58" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="E58" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="F58" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="G58" t="s">
-        <v>1374</v>
+        <v>995</v>
       </c>
       <c r="H58" t="s">
         <v>2</v>
@@ -41193,7 +41211,7 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
       <c r="B59" t="s">
         <v>1375</v>
@@ -41205,10 +41223,10 @@
         <v>1376</v>
       </c>
       <c r="E59" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="F59" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="G59" t="s">
         <v>1377</v>
@@ -41243,7 +41261,7 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
       <c r="B60" t="s">
         <v>1378</v>
@@ -41255,13 +41273,13 @@
         <v>1379</v>
       </c>
       <c r="E60" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="F60" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="G60" t="s">
-        <v>1016</v>
+        <v>1380</v>
       </c>
       <c r="H60" t="s">
         <v>2</v>
@@ -41293,25 +41311,25 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="B61" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="C61" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="D61" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="E61" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="F61" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="G61" t="s">
-        <v>1019</v>
+        <v>1383</v>
       </c>
       <c r="H61" t="s">
         <v>2</v>
@@ -41343,25 +41361,25 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="B62" t="s">
-        <v>1382</v>
+        <v>1384</v>
       </c>
       <c r="C62" t="s">
-        <v>1382</v>
+        <v>1384</v>
       </c>
       <c r="D62" t="s">
-        <v>1383</v>
+        <v>1385</v>
       </c>
       <c r="E62" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="F62" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="G62" t="s">
-        <v>1384</v>
+        <v>1016</v>
       </c>
       <c r="H62" t="s">
         <v>2</v>
@@ -41393,25 +41411,25 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="B63" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="C63" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="D63" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
       <c r="E63" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="F63" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="G63" t="s">
-        <v>1027</v>
+        <v>1019</v>
       </c>
       <c r="H63" t="s">
         <v>2</v>
@@ -41443,25 +41461,25 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="B64" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="C64" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="D64" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
       <c r="E64" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="F64" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="G64" t="s">
-        <v>1031</v>
+        <v>1390</v>
       </c>
       <c r="H64" t="s">
         <v>2</v>
@@ -41493,25 +41511,25 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="B65" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
       <c r="C65" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
       <c r="D65" t="s">
-        <v>1390</v>
+        <v>1392</v>
       </c>
       <c r="E65" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="F65" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="G65" t="s">
-        <v>1031</v>
+        <v>1027</v>
       </c>
       <c r="H65" t="s">
         <v>2</v>
@@ -41543,25 +41561,25 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
       <c r="B66" t="s">
-        <v>1391</v>
+        <v>1393</v>
       </c>
       <c r="C66" t="s">
-        <v>1391</v>
+        <v>1393</v>
       </c>
       <c r="D66" t="s">
-        <v>1392</v>
+        <v>1394</v>
       </c>
       <c r="E66" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="F66" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="G66" t="s">
-        <v>1037</v>
+        <v>1031</v>
       </c>
       <c r="H66" t="s">
         <v>2</v>
@@ -41593,25 +41611,25 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>438</v>
+        <v>430</v>
       </c>
       <c r="B67" t="s">
-        <v>1393</v>
+        <v>1395</v>
       </c>
       <c r="C67" t="s">
-        <v>1393</v>
+        <v>1395</v>
       </c>
       <c r="D67" t="s">
-        <v>1394</v>
+        <v>1396</v>
       </c>
       <c r="E67" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="F67" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="G67" t="s">
-        <v>1040</v>
+        <v>1031</v>
       </c>
       <c r="H67" t="s">
         <v>2</v>
@@ -41643,25 +41661,25 @@
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>442</v>
+        <v>434</v>
       </c>
       <c r="B68" t="s">
-        <v>1395</v>
+        <v>1397</v>
       </c>
       <c r="C68" t="s">
-        <v>1395</v>
+        <v>1397</v>
       </c>
       <c r="D68" t="s">
-        <v>1396</v>
+        <v>1398</v>
       </c>
       <c r="E68" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
       <c r="F68" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="G68" t="s">
-        <v>1044</v>
+        <v>1037</v>
       </c>
       <c r="H68" t="s">
         <v>2</v>
@@ -41693,25 +41711,25 @@
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
       <c r="B69" t="s">
-        <v>1397</v>
+        <v>1399</v>
       </c>
       <c r="C69" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="D69" t="s">
-        <v>1399</v>
+        <v>1400</v>
       </c>
       <c r="E69" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="F69" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="G69" t="s">
-        <v>1047</v>
+        <v>1040</v>
       </c>
       <c r="H69" t="s">
         <v>2</v>
@@ -41743,10 +41761,10 @@
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="B70" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="C70" t="s">
         <v>1401</v>
@@ -41755,13 +41773,13 @@
         <v>1402</v>
       </c>
       <c r="E70" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="F70" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
       <c r="G70" t="s">
-        <v>1403</v>
+        <v>1044</v>
       </c>
       <c r="H70" t="s">
         <v>2</v>
@@ -41782,36 +41800,36 @@
         <v>2</v>
       </c>
       <c r="N70" t="s">
-        <v>1253</v>
+        <v>2</v>
       </c>
       <c r="O70" t="s">
         <v>29</v>
       </c>
       <c r="P70" t="s">
-        <v>492</v>
+        <v>959</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>461</v>
+        <v>446</v>
       </c>
       <c r="B71" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C71" t="s">
         <v>1404</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>1405</v>
       </c>
-      <c r="D71" t="s">
-        <v>1406</v>
-      </c>
       <c r="E71" t="s">
-        <v>457</v>
+        <v>443</v>
       </c>
       <c r="F71" t="s">
-        <v>459</v>
+        <v>445</v>
       </c>
       <c r="G71" t="s">
-        <v>1407</v>
+        <v>1047</v>
       </c>
       <c r="H71" t="s">
         <v>2</v>
@@ -41832,36 +41850,36 @@
         <v>2</v>
       </c>
       <c r="N71" t="s">
-        <v>1253</v>
+        <v>2</v>
       </c>
       <c r="O71" t="s">
         <v>29</v>
       </c>
       <c r="P71" t="s">
-        <v>492</v>
+        <v>959</v>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>466</v>
+        <v>450</v>
       </c>
       <c r="B72" t="s">
+        <v>1406</v>
+      </c>
+      <c r="C72" t="s">
+        <v>1407</v>
+      </c>
+      <c r="D72" t="s">
         <v>1408</v>
       </c>
-      <c r="C72" t="s">
+      <c r="E72" t="s">
+        <v>447</v>
+      </c>
+      <c r="F72" t="s">
+        <v>449</v>
+      </c>
+      <c r="G72" t="s">
         <v>1409</v>
-      </c>
-      <c r="D72" t="s">
-        <v>1410</v>
-      </c>
-      <c r="E72" t="s">
-        <v>463</v>
-      </c>
-      <c r="F72" t="s">
-        <v>465</v>
-      </c>
-      <c r="G72" t="s">
-        <v>1411</v>
       </c>
       <c r="H72" t="s">
         <v>2</v>
@@ -41888,6 +41906,106 @@
         <v>29</v>
       </c>
       <c r="P72" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>461</v>
+      </c>
+      <c r="B73" t="s">
+        <v>1410</v>
+      </c>
+      <c r="C73" t="s">
+        <v>1411</v>
+      </c>
+      <c r="D73" t="s">
+        <v>1412</v>
+      </c>
+      <c r="E73" t="s">
+        <v>457</v>
+      </c>
+      <c r="F73" t="s">
+        <v>459</v>
+      </c>
+      <c r="G73" t="s">
+        <v>1413</v>
+      </c>
+      <c r="H73" t="s">
+        <v>2</v>
+      </c>
+      <c r="I73" t="s">
+        <v>2</v>
+      </c>
+      <c r="J73" t="s">
+        <v>2</v>
+      </c>
+      <c r="K73" t="s">
+        <v>2</v>
+      </c>
+      <c r="L73" t="s">
+        <v>2</v>
+      </c>
+      <c r="M73" t="s">
+        <v>2</v>
+      </c>
+      <c r="N73" t="s">
+        <v>1253</v>
+      </c>
+      <c r="O73" t="s">
+        <v>29</v>
+      </c>
+      <c r="P73" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>466</v>
+      </c>
+      <c r="B74" t="s">
+        <v>1414</v>
+      </c>
+      <c r="C74" t="s">
+        <v>1415</v>
+      </c>
+      <c r="D74" t="s">
+        <v>1416</v>
+      </c>
+      <c r="E74" t="s">
+        <v>463</v>
+      </c>
+      <c r="F74" t="s">
+        <v>465</v>
+      </c>
+      <c r="G74" t="s">
+        <v>1417</v>
+      </c>
+      <c r="H74" t="s">
+        <v>2</v>
+      </c>
+      <c r="I74" t="s">
+        <v>2</v>
+      </c>
+      <c r="J74" t="s">
+        <v>2</v>
+      </c>
+      <c r="K74" t="s">
+        <v>2</v>
+      </c>
+      <c r="L74" t="s">
+        <v>2</v>
+      </c>
+      <c r="M74" t="s">
+        <v>2</v>
+      </c>
+      <c r="N74" t="s">
+        <v>1253</v>
+      </c>
+      <c r="O74" t="s">
+        <v>29</v>
+      </c>
+      <c r="P74" t="s">
         <v>492</v>
       </c>
     </row>
@@ -41900,7 +42018,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -41927,7 +42045,7 @@
         <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1412</v>
+        <v>1418</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>21</v>
@@ -42096,22 +42214,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
         <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="D9" t="s">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="E9" t="s">
         <v>37</v>
       </c>
       <c r="F9">
-        <v>18.6</v>
+        <v>17.8</v>
       </c>
       <c r="G9" t="s">
         <v>30</v>
@@ -42119,22 +42237,22 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="B10" t="s">
         <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E10" t="s">
         <v>37</v>
       </c>
       <c r="F10">
-        <v>17.8</v>
+        <v>16</v>
       </c>
       <c r="G10" t="s">
         <v>30</v>
@@ -42142,22 +42260,22 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>144</v>
       </c>
       <c r="B11" t="s">
         <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="D11" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
       <c r="E11" t="s">
         <v>37</v>
       </c>
       <c r="F11">
-        <v>16</v>
+        <v>13.9</v>
       </c>
       <c r="G11" t="s">
         <v>30</v>
@@ -42165,16 +42283,16 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D12" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E12" t="s">
         <v>37</v>
@@ -42188,22 +42306,22 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>148</v>
+        <v>121</v>
       </c>
       <c r="D13" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="E13" t="s">
         <v>37</v>
       </c>
       <c r="F13">
-        <v>13.9</v>
+        <v>12.3</v>
       </c>
       <c r="G13" t="s">
         <v>30</v>
@@ -42211,19 +42329,19 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>120</v>
+        <v>283</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>284</v>
       </c>
       <c r="C14" t="s">
-        <v>121</v>
+        <v>285</v>
       </c>
       <c r="D14" t="s">
-        <v>123</v>
+        <v>287</v>
       </c>
       <c r="E14" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F14">
         <v>12.3</v>
@@ -42234,22 +42352,22 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>283</v>
+        <v>154</v>
       </c>
       <c r="B15" t="s">
-        <v>284</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>285</v>
+        <v>155</v>
       </c>
       <c r="D15" t="s">
-        <v>287</v>
+        <v>157</v>
       </c>
       <c r="E15" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F15">
-        <v>12.3</v>
+        <v>10.3</v>
       </c>
       <c r="G15" t="s">
         <v>30</v>
@@ -42257,16 +42375,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>154</v>
+        <v>303</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>304</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>305</v>
       </c>
       <c r="D16" t="s">
-        <v>157</v>
+        <v>306</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
@@ -42275,24 +42393,24 @@
         <v>10.3</v>
       </c>
       <c r="G16" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>303</v>
+        <v>447</v>
       </c>
       <c r="B17" t="s">
-        <v>304</v>
+        <v>448</v>
       </c>
       <c r="C17" t="s">
-        <v>305</v>
+        <v>449</v>
       </c>
       <c r="D17" t="s">
-        <v>306</v>
+        <v>450</v>
       </c>
       <c r="E17" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F17">
         <v>10.3</v>
@@ -42303,68 +42421,68 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>447</v>
+        <v>273</v>
       </c>
       <c r="B18" t="s">
-        <v>448</v>
+        <v>274</v>
       </c>
       <c r="C18" t="s">
-        <v>449</v>
+        <v>275</v>
       </c>
       <c r="D18" t="s">
-        <v>450</v>
+        <v>143</v>
       </c>
       <c r="E18" t="s">
         <v>183</v>
       </c>
       <c r="F18">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>307</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>273</v>
+        <v>308</v>
       </c>
       <c r="B19" t="s">
-        <v>274</v>
+        <v>304</v>
       </c>
       <c r="C19" t="s">
-        <v>275</v>
+        <v>309</v>
       </c>
       <c r="D19" t="s">
-        <v>143</v>
+        <v>311</v>
       </c>
       <c r="E19" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F19">
-        <v>10</v>
+        <v>9.8</v>
       </c>
       <c r="G19" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="B20" t="s">
         <v>304</v>
       </c>
       <c r="C20" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D20" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="E20" t="s">
         <v>37</v>
       </c>
       <c r="F20">
-        <v>9.8</v>
+        <v>9.3</v>
       </c>
       <c r="G20" t="s">
         <v>307</v>
@@ -42372,108 +42490,108 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>312</v>
+        <v>158</v>
       </c>
       <c r="B21" t="s">
-        <v>304</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>313</v>
+        <v>159</v>
       </c>
       <c r="D21" t="s">
-        <v>315</v>
+        <v>161</v>
       </c>
       <c r="E21" t="s">
         <v>37</v>
       </c>
       <c r="F21">
-        <v>9.3</v>
+        <v>9</v>
       </c>
       <c r="G21" t="s">
-        <v>307</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>316</v>
+        <v>179</v>
       </c>
       <c r="B22" t="s">
-        <v>304</v>
+        <v>180</v>
       </c>
       <c r="C22" t="s">
-        <v>317</v>
+        <v>181</v>
       </c>
       <c r="D22" t="s">
-        <v>318</v>
+        <v>182</v>
       </c>
       <c r="E22" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F22">
-        <v>9.3</v>
+        <v>8.3</v>
       </c>
       <c r="G22" t="s">
-        <v>307</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>158</v>
+        <v>335</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>304</v>
       </c>
       <c r="C23" t="s">
-        <v>159</v>
+        <v>336</v>
       </c>
       <c r="D23" t="s">
-        <v>161</v>
+        <v>337</v>
       </c>
       <c r="E23" t="s">
         <v>37</v>
       </c>
       <c r="F23">
-        <v>9</v>
+        <v>8.3</v>
       </c>
       <c r="G23" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>179</v>
+        <v>341</v>
       </c>
       <c r="B24" t="s">
-        <v>180</v>
+        <v>304</v>
       </c>
       <c r="C24" t="s">
-        <v>181</v>
+        <v>342</v>
       </c>
       <c r="D24" t="s">
-        <v>182</v>
+        <v>343</v>
       </c>
       <c r="E24" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F24">
         <v>8.3</v>
       </c>
       <c r="G24" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="B25" t="s">
         <v>304</v>
       </c>
       <c r="C25" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="D25" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="E25" t="s">
         <v>37</v>
@@ -42487,108 +42605,108 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>341</v>
+        <v>267</v>
       </c>
       <c r="B26" t="s">
-        <v>304</v>
+        <v>268</v>
       </c>
       <c r="C26" t="s">
-        <v>342</v>
+        <v>269</v>
       </c>
       <c r="D26" t="s">
-        <v>343</v>
+        <v>193</v>
       </c>
       <c r="E26" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F26">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G26" t="s">
-        <v>307</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>344</v>
+        <v>270</v>
       </c>
       <c r="B27" t="s">
-        <v>304</v>
+        <v>271</v>
       </c>
       <c r="C27" t="s">
-        <v>345</v>
+        <v>272</v>
       </c>
       <c r="D27" t="s">
-        <v>346</v>
+        <v>247</v>
       </c>
       <c r="E27" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F27">
-        <v>8.3</v>
+        <v>8</v>
       </c>
       <c r="G27" t="s">
-        <v>307</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>267</v>
+        <v>353</v>
       </c>
       <c r="B28" t="s">
-        <v>268</v>
+        <v>304</v>
       </c>
       <c r="C28" t="s">
-        <v>269</v>
+        <v>354</v>
       </c>
       <c r="D28" t="s">
-        <v>193</v>
+        <v>355</v>
       </c>
       <c r="E28" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F28">
         <v>8</v>
       </c>
       <c r="G28" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>270</v>
+        <v>356</v>
       </c>
       <c r="B29" t="s">
-        <v>271</v>
+        <v>304</v>
       </c>
       <c r="C29" t="s">
-        <v>272</v>
+        <v>357</v>
       </c>
       <c r="D29" t="s">
-        <v>247</v>
+        <v>358</v>
       </c>
       <c r="E29" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="F29">
         <v>8</v>
       </c>
       <c r="G29" t="s">
-        <v>30</v>
+        <v>307</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B30" t="s">
         <v>304</v>
       </c>
       <c r="C30" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="D30" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="E30" t="s">
         <v>37</v>
@@ -42602,16 +42720,16 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="B31" t="s">
         <v>304</v>
       </c>
       <c r="C31" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="D31" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="E31" t="s">
         <v>37</v>
@@ -42625,16 +42743,16 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B32" t="s">
         <v>304</v>
       </c>
       <c r="C32" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="D32" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="E32" t="s">
         <v>37</v>
@@ -42648,70 +42766,24 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>362</v>
+        <v>276</v>
       </c>
       <c r="B33" t="s">
-        <v>304</v>
+        <v>277</v>
       </c>
       <c r="C33" t="s">
-        <v>363</v>
+        <v>278</v>
       </c>
       <c r="D33" t="s">
-        <v>364</v>
+        <v>2</v>
       </c>
       <c r="E33" t="s">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="F33">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="G33" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>365</v>
-      </c>
-      <c r="B34" t="s">
-        <v>304</v>
-      </c>
-      <c r="C34" t="s">
-        <v>366</v>
-      </c>
-      <c r="D34" t="s">
-        <v>367</v>
-      </c>
-      <c r="E34" t="s">
-        <v>37</v>
-      </c>
-      <c r="F34">
-        <v>8</v>
-      </c>
-      <c r="G34" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>276</v>
-      </c>
-      <c r="B35" t="s">
-        <v>277</v>
-      </c>
-      <c r="C35" t="s">
-        <v>278</v>
-      </c>
-      <c r="D35" t="s">
-        <v>2</v>
-      </c>
-      <c r="E35" t="s">
-        <v>183</v>
-      </c>
-      <c r="F35">
-        <v>0.8</v>
-      </c>
-      <c r="G35" t="s">
         <v>30</v>
       </c>
     </row>
@@ -42818,27 +42890,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>1413</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1414</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1415</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1416</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1417</v>
+        <v>1423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>